<commit_message>
feat: implement wine synchronization and 'Add Wine' UI component
</commit_message>
<xml_diff>
--- a/Weinlager_Details.xlsx
+++ b/Weinlager_Details.xlsx
@@ -405,7 +405,7 @@
     <col min="4" max="4" width="15.83203125" customWidth="1"/>
     <col min="5" max="5" width="37.83203125" customWidth="1"/>
     <col min="6" max="6" width="17.83203125" customWidth="1"/>
-    <col min="7" max="7" width="122.83203125" customWidth="1"/>
+    <col min="7" max="7" width="49.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -681,7 +681,7 @@
         <v/>
       </c>
       <c r="G12" t="str">
-        <v>Säuerlich und fad</v>
+        <v/>
       </c>
     </row>
     <row r="13">
@@ -727,7 +727,7 @@
         <v/>
       </c>
       <c r="G14" t="str">
-        <v>Gute Nase, cremig, kein Holz, schmackhaft</v>
+        <v/>
       </c>
     </row>
     <row r="15">
@@ -796,7 +796,7 @@
         <v/>
       </c>
       <c r="G17" t="str">
-        <v>Auch besser am nächsten Tag. leichte Frucht, süffig, aber bisschen fad</v>
+        <v/>
       </c>
     </row>
     <row r="18">
@@ -819,7 +819,7 @@
         <v/>
       </c>
       <c r="G18" t="str">
-        <v>Besser am nächsten Tag. Musste atmen. Erster Eindruck Frucht, dann kommt die Säure</v>
+        <v/>
       </c>
     </row>
     <row r="19">
@@ -957,7 +957,7 @@
         <v/>
       </c>
       <c r="G24" t="str">
-        <v>Fruchtig bezaubernde Nase. Holznote, deutliche Säure, frisch, nicht zu schwer, gut ausbalanciert. Positive Überraschung!</v>
+        <v/>
       </c>
     </row>
     <row r="25">
@@ -1003,7 +1003,7 @@
         <v/>
       </c>
       <c r="G26" t="str">
-        <v>Preiswert. Fruchtige Nase. Harmonische Säure. Guter Alltagswein</v>
+        <v/>
       </c>
     </row>
     <row r="27">
@@ -1026,7 +1026,7 @@
         <v/>
       </c>
       <c r="G27" t="str">
-        <v>Uninteressant</v>
+        <v/>
       </c>
     </row>
     <row r="28">
@@ -1049,7 +1049,7 @@
         <v/>
       </c>
       <c r="G28" t="str">
-        <v>relativ langweilig</v>
+        <v/>
       </c>
     </row>
     <row r="29">
@@ -1072,7 +1072,7 @@
         <v/>
       </c>
       <c r="G29" t="str">
-        <v>Vanillenote, wenig Säure, harmonisch</v>
+        <v/>
       </c>
     </row>
     <row r="30">
@@ -1736,10 +1736,10 @@
         <v>fruchtbetont</v>
       </c>
       <c r="F58" t="str">
-        <v>★★★★</v>
+        <v/>
       </c>
       <c r="G58" t="str">
-        <v>Schwarz Mainburg gut trinkbar</v>
+        <v/>
       </c>
     </row>
     <row r="59">
@@ -1759,10 +1759,10 @@
         <v>leicht &amp; fruchtbetont</v>
       </c>
       <c r="F59" t="str">
-        <v>★★</v>
+        <v/>
       </c>
       <c r="G59" t="str">
-        <v>Schwarz Mainburg 11,90 deutlich teurer, aber nichts besonderes</v>
+        <v/>
       </c>
     </row>
     <row r="60">
@@ -1782,10 +1782,10 @@
         <v>elegant &amp; beerig</v>
       </c>
       <c r="F60" t="str">
-        <v>★★★</v>
+        <v/>
       </c>
       <c r="G60" t="str">
-        <v>Okay</v>
+        <v/>
       </c>
     </row>
     <row r="61">
@@ -1805,10 +1805,10 @@
         <v>strukturiert &amp; fruchtig</v>
       </c>
       <c r="F61" t="str">
-        <v>★★★</v>
+        <v/>
       </c>
       <c r="G61" t="str">
-        <v>Not bad</v>
+        <v/>
       </c>
     </row>
     <row r="62">
@@ -1828,10 +1828,10 @@
         <v>fruchtbetont</v>
       </c>
       <c r="F62" t="str">
-        <v>★★★★★</v>
+        <v/>
       </c>
       <c r="G62" t="str">
-        <v>Sehr gut für den Preis</v>
+        <v/>
       </c>
     </row>
     <row r="63">
@@ -1851,10 +1851,10 @@
         <v>kräftig &amp; würzig</v>
       </c>
       <c r="F63" t="str">
-        <v>★★★★</v>
+        <v/>
       </c>
       <c r="G63" t="str">
-        <v>Gut um 6€</v>
+        <v/>
       </c>
     </row>
     <row r="64">
@@ -1874,10 +1874,10 @@
         <v>ausgewogen</v>
       </c>
       <c r="F64" t="str">
-        <v>★★★★★</v>
+        <v/>
       </c>
       <c r="G64" t="str">
-        <v>Von der Gemeinschaft für lecker befunden</v>
+        <v/>
       </c>
     </row>
     <row r="65">
@@ -1897,10 +1897,10 @@
         <v>fruchtig</v>
       </c>
       <c r="F65" t="str">
-        <v>★★★★</v>
+        <v/>
       </c>
       <c r="G65" t="str">
-        <v>Gut</v>
+        <v/>
       </c>
     </row>
     <row r="66">
@@ -1920,10 +1920,10 @@
         <v>elegant &amp; mineralisch</v>
       </c>
       <c r="F66" t="str">
-        <v>★★★★</v>
+        <v/>
       </c>
       <c r="G66" t="str">
-        <v>Demeter Restaurant Gut</v>
+        <v/>
       </c>
     </row>
     <row r="67">
@@ -1943,10 +1943,10 @@
         <v>fruchtbetont</v>
       </c>
       <c r="F67" t="str">
-        <v>★★</v>
+        <v/>
       </c>
       <c r="G67" t="str">
-        <v>Schwarz Mainburg nichts besonderes</v>
+        <v/>
       </c>
     </row>
     <row r="68">
@@ -1969,7 +1969,7 @@
         <v/>
       </c>
       <c r="G68" t="str">
-        <v>Weinland Giesing Safferts Winzer Welt süffig, bisschen süß</v>
+        <v/>
       </c>
     </row>
     <row r="69">
@@ -1989,10 +1989,10 @@
         <v>fruchtig</v>
       </c>
       <c r="F69" t="str">
-        <v>★★★★</v>
+        <v/>
       </c>
       <c r="G69" t="str">
-        <v>Weinberg Giesing Um 10€ gut, aber nichts besonderes</v>
+        <v/>
       </c>
     </row>
     <row r="70">
@@ -2015,7 +2015,7 @@
         <v/>
       </c>
       <c r="G70" t="str">
-        <v>Weinberg. Süßlich mit Säure und Holznote. Eigenwillig, aber teuer</v>
+        <v/>
       </c>
     </row>
     <row r="71">
@@ -2035,10 +2035,10 @@
         <v>kräftig &amp; strukturiert</v>
       </c>
       <c r="F71" t="str">
-        <v>★★★</v>
+        <v/>
       </c>
       <c r="G71" t="str">
-        <v>Nicht schlecht aber zu teuer</v>
+        <v/>
       </c>
     </row>
     <row r="72">
@@ -2058,10 +2058,10 @@
         <v>schwer &amp; süßlich</v>
       </c>
       <c r="F72" t="str">
-        <v>★</v>
+        <v/>
       </c>
       <c r="G72" t="str">
-        <v>Schwarz. Sehr schwer, süßlich, nicht empfehlenswert</v>
+        <v/>
       </c>
     </row>
     <row r="73">
@@ -2081,10 +2081,10 @@
         <v>fruchtig (Bio)</v>
       </c>
       <c r="F73" t="str">
-        <v>★★★★★</v>
+        <v/>
       </c>
       <c r="G73" t="str">
-        <v>Preiswert gut Super U</v>
+        <v/>
       </c>
     </row>
     <row r="74">
@@ -2104,10 +2104,10 @@
         <v>beerig &amp; ausgewogen</v>
       </c>
       <c r="F74" t="str">
-        <v>★★</v>
+        <v/>
       </c>
       <c r="G74" t="str">
-        <v>Billig, aber nichts besonderes</v>
+        <v/>
       </c>
     </row>
     <row r="75">
@@ -2127,10 +2127,10 @@
         <v>fruchtig &amp; würzig</v>
       </c>
       <c r="F75" t="str">
-        <v>★★★★</v>
+        <v/>
       </c>
       <c r="G75" t="str">
-        <v>Holz und gute Frucht Säure Balance. Preiswert</v>
+        <v/>
       </c>
     </row>
     <row r="76">
@@ -2150,10 +2150,10 @@
         <v>frisch &amp; aromatisch</v>
       </c>
       <c r="F76" t="str">
-        <v>★★★★★</v>
+        <v/>
       </c>
       <c r="G76" t="str">
-        <v>Super U interessantes Holz Aroma. Süffig!</v>
+        <v/>
       </c>
     </row>
     <row r="77">
@@ -2173,10 +2173,10 @@
         <v>beerig &amp; weich</v>
       </c>
       <c r="F77" t="str">
-        <v>★★★★★</v>
+        <v/>
       </c>
       <c r="G77" t="str">
-        <v>Super U nichts mehr</v>
+        <v/>
       </c>
     </row>
     <row r="78">
@@ -2196,10 +2196,10 @@
         <v>strukturiert &amp; holzig</v>
       </c>
       <c r="F78" t="str">
-        <v>★</v>
+        <v/>
       </c>
       <c r="G78" t="str">
-        <v>Nicht empfehlenswert</v>
+        <v/>
       </c>
     </row>
     <row r="79">
@@ -2219,10 +2219,10 @@
         <v>fruchtig (Bio)</v>
       </c>
       <c r="F79" t="str">
-        <v>★★★</v>
+        <v/>
       </c>
       <c r="G79" t="str">
-        <v>Okay</v>
+        <v/>
       </c>
     </row>
     <row r="80">
@@ -2242,10 +2242,10 @@
         <v>strukturiert &amp; würzig</v>
       </c>
       <c r="F80" t="str">
-        <v>★★★★</v>
+        <v/>
       </c>
       <c r="G80" t="str">
-        <v>Gut</v>
+        <v/>
       </c>
     </row>
     <row r="81">
@@ -2265,10 +2265,10 @@
         <v>beerig &amp; mineralisch</v>
       </c>
       <c r="F81" t="str">
-        <v>★★★★</v>
+        <v/>
       </c>
       <c r="G81" t="str">
-        <v>Gut am zweiten Tag</v>
+        <v/>
       </c>
     </row>
     <row r="82">
@@ -2288,10 +2288,10 @@
         <v>intensiv &amp; barrique</v>
       </c>
       <c r="F82" t="str">
-        <v>★★★★</v>
+        <v/>
       </c>
       <c r="G82" t="str">
-        <v>Barrique, intensiv, gut!</v>
+        <v/>
       </c>
     </row>
     <row r="83">
@@ -2311,10 +2311,10 @@
         <v>elegant &amp; würzig</v>
       </c>
       <c r="F83" t="str">
-        <v>★</v>
+        <v/>
       </c>
       <c r="G83" t="str">
-        <v>Sauer, nicht herausragend</v>
+        <v/>
       </c>
     </row>
     <row r="84">
@@ -2334,10 +2334,10 @@
         <v>ausgewogen &amp; beerig</v>
       </c>
       <c r="F84" t="str">
-        <v>★★★★</v>
+        <v/>
       </c>
       <c r="G84" t="str">
-        <v>Auch nicht gut</v>
+        <v/>
       </c>
     </row>
     <row r="85">
@@ -2380,10 +2380,10 @@
         <v>fruchtig &amp; würzig</v>
       </c>
       <c r="F86" t="str">
-        <v>★★★</v>
+        <v/>
       </c>
       <c r="G86" t="str">
-        <v>Säuerlich, aber nicht schlecht</v>
+        <v/>
       </c>
     </row>
     <row r="87">
@@ -2403,10 +2403,10 @@
         <v>fruchtig &amp; klassisch</v>
       </c>
       <c r="F87" t="str">
-        <v>★★★★</v>
+        <v/>
       </c>
       <c r="G87" t="str">
-        <v>Gut</v>
+        <v/>
       </c>
     </row>
     <row r="88">
@@ -2426,10 +2426,10 @@
         <v>elegant &amp; beerig</v>
       </c>
       <c r="F88" t="str">
-        <v>★★★</v>
+        <v/>
       </c>
       <c r="G88" t="str">
-        <v>Okay</v>
+        <v/>
       </c>
     </row>
     <row r="89">
@@ -2449,10 +2449,10 @@
         <v>intensiv &amp; barrique</v>
       </c>
       <c r="F89" t="str">
-        <v>★★★★</v>
+        <v/>
       </c>
       <c r="G89" t="str">
-        <v>Barrique, intensiv, gut</v>
+        <v/>
       </c>
     </row>
     <row r="90">
@@ -2472,10 +2472,10 @@
         <v>kräftig &amp; beerig</v>
       </c>
       <c r="F90" t="str">
-        <v>★★★★★</v>
+        <v/>
       </c>
       <c r="G90" t="str">
-        <v>Sehr gut</v>
+        <v/>
       </c>
     </row>
     <row r="91">
@@ -2495,10 +2495,10 @@
         <v>klassisch &amp; beerig</v>
       </c>
       <c r="F91" t="str">
-        <v>★★★★★</v>
+        <v/>
       </c>
       <c r="G91" t="str">
-        <v>Nicht Super</v>
+        <v/>
       </c>
     </row>
     <row r="92">
@@ -2518,10 +2518,10 @@
         <v>beerig &amp; holzig</v>
       </c>
       <c r="F92" t="str">
-        <v>★★★★</v>
+        <v/>
       </c>
       <c r="G92" t="str">
-        <v>Gut</v>
+        <v/>
       </c>
     </row>
     <row r="93">
@@ -2541,10 +2541,10 @@
         <v>frisch &amp; mediterran (Bio)</v>
       </c>
       <c r="F93" t="str">
-        <v>★★</v>
+        <v/>
       </c>
       <c r="G93" t="str">
-        <v>langweilig</v>
+        <v/>
       </c>
     </row>
     <row r="94">
@@ -2564,10 +2564,10 @@
         <v>einfach &amp; süffig</v>
       </c>
       <c r="F94" t="str">
-        <v>★★★</v>
+        <v/>
       </c>
       <c r="G94" t="str">
-        <v>ok</v>
+        <v/>
       </c>
     </row>
     <row r="95">
@@ -2587,10 +2587,10 @@
         <v>leicht &amp; säurebetont</v>
       </c>
       <c r="F95" t="str">
-        <v>★★★★</v>
+        <v/>
       </c>
       <c r="G95" t="str">
-        <v>leicht und gut</v>
+        <v/>
       </c>
     </row>
     <row r="96">
@@ -2613,7 +2613,7 @@
         <v/>
       </c>
       <c r="G96" t="str">
-        <v>nicht herausragend</v>
+        <v/>
       </c>
     </row>
     <row r="97">
@@ -2633,10 +2633,10 @@
         <v>intensiv &amp; fruchtig (Bio)</v>
       </c>
       <c r="F97" t="str">
-        <v>★★★</v>
+        <v/>
       </c>
       <c r="G97" t="str">
-        <v>okay</v>
+        <v/>
       </c>
     </row>
     <row r="98">
@@ -2656,10 +2656,10 @@
         <v>fruchtig &amp; weich</v>
       </c>
       <c r="F98" t="str">
-        <v>★★★</v>
+        <v/>
       </c>
       <c r="G98" t="str">
-        <v>Ok</v>
+        <v/>
       </c>
     </row>
     <row r="99">
@@ -2679,10 +2679,10 @@
         <v>elegant &amp; fruchtig</v>
       </c>
       <c r="F99" t="str">
-        <v>★★★</v>
+        <v/>
       </c>
       <c r="G99" t="str">
-        <v>Ok</v>
+        <v/>
       </c>
     </row>
     <row r="100">
@@ -2705,7 +2705,7 @@
         <v/>
       </c>
       <c r="G100" t="str">
-        <v>Barrique, aber nicht herausragend</v>
+        <v/>
       </c>
     </row>
     <row r="101">
@@ -2725,10 +2725,10 @@
         <v>strukturiert (Bio)</v>
       </c>
       <c r="F101" t="str">
-        <v>★★</v>
+        <v/>
       </c>
       <c r="G101" t="str">
-        <v>Säuerlich, fad</v>
+        <v/>
       </c>
     </row>
     <row r="102">
@@ -2751,7 +2751,7 @@
         <v/>
       </c>
       <c r="G102" t="str">
-        <v>Leicht, nicht sehr komplex, Recht teuer</v>
+        <v/>
       </c>
     </row>
     <row r="103">
@@ -2771,10 +2771,10 @@
         <v>beerig &amp; vanillig</v>
       </c>
       <c r="F103" t="str">
-        <v>★★★</v>
+        <v/>
       </c>
       <c r="G103" t="str">
-        <v>Bisschen Vanille, ok</v>
+        <v/>
       </c>
     </row>
     <row r="104">
@@ -2794,10 +2794,10 @@
         <v>säurebetont &amp; natur</v>
       </c>
       <c r="F104" t="str">
-        <v>★★★★</v>
+        <v/>
       </c>
       <c r="G104" t="str">
-        <v>Spontanvergoren, typische Natur-Wein Säure, gut!</v>
+        <v/>
       </c>
     </row>
     <row r="105">
@@ -2817,10 +2817,10 @@
         <v>intensiv &amp; fruchtig</v>
       </c>
       <c r="F105" t="str">
-        <v>★★★★</v>
+        <v/>
       </c>
       <c r="G105" t="str">
-        <v>intensives Aroma, Geschmack gut, aber weniger intensiv</v>
+        <v/>
       </c>
     </row>
     <row r="106">
@@ -2840,10 +2840,10 @@
         <v>mineralisch &amp; fruchtig</v>
       </c>
       <c r="F106" t="str">
-        <v>★★★★★</v>
+        <v/>
       </c>
       <c r="G106" t="str">
-        <v>Sehr guter Weißwein!</v>
+        <v/>
       </c>
     </row>
     <row r="107">
@@ -2886,10 +2886,10 @@
         <v>beerig &amp; schokoladig</v>
       </c>
       <c r="F108" t="str">
-        <v>★★★</v>
+        <v/>
       </c>
       <c r="G108" t="str">
-        <v>Konventionell, Vanille, nicht schlecht</v>
+        <v/>
       </c>
     </row>
     <row r="109">
@@ -2909,10 +2909,10 @@
         <v>fruchtig &amp; klassisch</v>
       </c>
       <c r="F109" t="str">
-        <v>★★★</v>
+        <v/>
       </c>
       <c r="G109" t="str">
-        <v>ok</v>
+        <v/>
       </c>
     </row>
     <row r="110">
@@ -2932,10 +2932,10 @@
         <v>elegant &amp; fein</v>
       </c>
       <c r="F110" t="str">
-        <v>★★★★</v>
+        <v/>
       </c>
       <c r="G110" t="str">
-        <v>Gut Maische + Spontanvergoren</v>
+        <v/>
       </c>
     </row>
     <row r="111">
@@ -2955,10 +2955,10 @@
         <v>ausgewogen</v>
       </c>
       <c r="F111" t="str">
-        <v>★★★★</v>
+        <v/>
       </c>
       <c r="G111" t="str">
-        <v>gut</v>
+        <v/>
       </c>
     </row>
     <row r="112">
@@ -2978,10 +2978,10 @@
         <v>frisch &amp; pfeffrig</v>
       </c>
       <c r="F112" t="str">
-        <v>★★★★</v>
+        <v/>
       </c>
       <c r="G112" t="str">
-        <v>relativ preiswert gut trinkbar dezente Säure wenig Tiefe</v>
+        <v/>
       </c>
     </row>
     <row r="113">
@@ -3001,10 +3001,10 @@
         <v>fruchtig (Bio)</v>
       </c>
       <c r="F113" t="str">
-        <v>★★★</v>
+        <v/>
       </c>
       <c r="G113" t="str">
-        <v>ok, aber kein Kaufempfehlung</v>
+        <v/>
       </c>
     </row>
     <row r="114">
@@ -3027,7 +3027,7 @@
         <v/>
       </c>
       <c r="G114" t="str">
-        <v>Portugieser süffig, relativ preiswert</v>
+        <v/>
       </c>
     </row>
     <row r="115">
@@ -3050,7 +3050,7 @@
         <v/>
       </c>
       <c r="G115" t="str">
-        <v>aufdringliches Vanille Aroma. Geschmackssache!</v>
+        <v/>
       </c>
     </row>
     <row r="116">
@@ -3073,7 +3073,7 @@
         <v/>
       </c>
       <c r="G116" t="str">
-        <v>süffig preiswert</v>
+        <v/>
       </c>
     </row>
     <row r="117">
@@ -3096,7 +3096,7 @@
         <v/>
       </c>
       <c r="G117" t="str">
-        <v>süffig</v>
+        <v/>
       </c>
     </row>
     <row r="118">
@@ -3116,10 +3116,10 @@
         <v>kräftig &amp; fruchtig (Bio)</v>
       </c>
       <c r="F118" t="str">
-        <v>★★★★</v>
+        <v/>
       </c>
       <c r="G118" t="str">
-        <v>kräftig und schmackhaft</v>
+        <v/>
       </c>
     </row>
     <row r="119">
@@ -3142,7 +3142,7 @@
         <v/>
       </c>
       <c r="G119" t="str">
-        <v>leicht unangenehm marmeladig</v>
+        <v/>
       </c>
     </row>
     <row r="120">
@@ -3165,7 +3165,7 @@
         <v/>
       </c>
       <c r="G120" t="str">
-        <v>schön fruchtig süffig nicht zu süß</v>
+        <v/>
       </c>
     </row>
     <row r="121">
@@ -3188,7 +3188,7 @@
         <v/>
       </c>
       <c r="G121" t="str">
-        <v>Vanillenote, sonst recht schlicht</v>
+        <v/>
       </c>
     </row>
     <row r="122">
@@ -3208,10 +3208,10 @@
         <v>harmonisch &amp; leicht</v>
       </c>
       <c r="F122" t="str">
-        <v>★★★★</v>
+        <v/>
       </c>
       <c r="G122" t="str">
-        <v>Leichter Maischegeschmack. Harmonisch, rund</v>
+        <v/>
       </c>
     </row>
     <row r="123">
@@ -3231,10 +3231,10 @@
         <v>beerig &amp; würzig</v>
       </c>
       <c r="F123" t="str">
-        <v>★★★★</v>
+        <v/>
       </c>
       <c r="G123" t="str">
-        <v>Harmonisch, feine Würze, Charakter, leicht Barriquik, brendan sagt a bissl flach :)</v>
+        <v/>
       </c>
     </row>
     <row r="124">
@@ -3257,7 +3257,7 @@
         <v/>
       </c>
       <c r="G124" t="str">
-        <v>Leicht säuerlich, bei Zimmertemperatur Eindruck leichter Fehlnote</v>
+        <v/>
       </c>
     </row>
     <row r="125">
@@ -3280,7 +3280,7 @@
         <v/>
       </c>
       <c r="G125" t="str">
-        <v>Süffig, aber nicht sehr aromatisch</v>
+        <v/>
       </c>
     </row>
     <row r="126">
@@ -3300,10 +3300,10 @@
         <v>würzig &amp; beerig (Bio)</v>
       </c>
       <c r="F126" t="str">
-        <v>★★★</v>
+        <v/>
       </c>
       <c r="G126" t="str">
-        <v>Nicht schlecht</v>
+        <v/>
       </c>
     </row>
     <row r="127">
@@ -3326,7 +3326,7 @@
         <v/>
       </c>
       <c r="G127" t="str">
-        <v>Für den Preis 19,92 € / Bewertung (Lobenberg: 95/100 Parker: 93/100 Wine Spectator: 93/100) relativ unspektakulär</v>
+        <v/>
       </c>
     </row>
     <row r="128">
@@ -3346,10 +3346,10 @@
         <v>frisch &amp; fruchtig</v>
       </c>
       <c r="F128" t="str">
-        <v>★★★</v>
+        <v/>
       </c>
       <c r="G128" t="str">
-        <v>Leichte Frucht und Säure, süffig, preiswert, ok</v>
+        <v/>
       </c>
     </row>
     <row r="129">
@@ -3372,7 +3372,7 @@
         <v/>
       </c>
       <c r="G129" t="str">
-        <v>Trocken, wenig Frucht, nicht besonders aromatisch, süffig</v>
+        <v/>
       </c>
     </row>
     <row r="130">
@@ -3392,10 +3392,10 @@
         <v>harmonisch &amp; intensiv</v>
       </c>
       <c r="F130" t="str">
-        <v>★★★★</v>
+        <v/>
       </c>
       <c r="G130" t="str">
-        <v>Harmonisch, intensiv, preiswert, gut</v>
+        <v/>
       </c>
     </row>
     <row r="131">
@@ -3415,10 +3415,10 @@
         <v>harmonisch &amp; fruchtig</v>
       </c>
       <c r="F131" t="str">
-        <v>★★★★</v>
+        <v/>
       </c>
       <c r="G131" t="str">
-        <v>Harmonisch, vielschichtig mit leichtem Barrique</v>
+        <v/>
       </c>
     </row>
     <row r="132">
@@ -3438,10 +3438,10 @@
         <v>fruchtig (Bio)</v>
       </c>
       <c r="F132" t="str">
-        <v>★★</v>
+        <v/>
       </c>
       <c r="G132" t="str">
-        <v>Nase unauffällig, leicht säuerlich und flach</v>
+        <v/>
       </c>
     </row>
     <row r="133">
@@ -3464,7 +3464,7 @@
         <v/>
       </c>
       <c r="G133" t="str">
-        <v>Leicht säuerlich, recht flach</v>
+        <v/>
       </c>
     </row>
     <row r="134">
@@ -3487,7 +3487,7 @@
         <v/>
       </c>
       <c r="G134" t="str">
-        <v>Leicht marmeladig, etwas besser, aber auch nicht berauschend</v>
+        <v/>
       </c>
     </row>
     <row r="135">
@@ -3510,7 +3510,7 @@
         <v/>
       </c>
       <c r="G135" t="str">
-        <v>Schwer zu beschreibende Note. Fehlnote, viel Tannin oder lange auf der Maische?</v>
+        <v/>
       </c>
     </row>
     <row r="136">
@@ -3530,10 +3530,10 @@
         <v>harmonisch</v>
       </c>
       <c r="F136" t="str">
-        <v>★★★★</v>
+        <v/>
       </c>
       <c r="G136" t="str">
-        <v>Gut trinkbar, harmonisch, aber unauffällig</v>
+        <v/>
       </c>
     </row>
     <row r="137">
@@ -3553,10 +3553,10 @@
         <v>beerig &amp; weich</v>
       </c>
       <c r="F137" t="str">
-        <v>★★</v>
+        <v/>
       </c>
       <c r="G137" t="str">
-        <v>Unauffällig</v>
+        <v/>
       </c>
     </row>
     <row r="138">
@@ -3576,10 +3576,10 @@
         <v>samtig &amp; weich</v>
       </c>
       <c r="F138" t="str">
-        <v>★★</v>
+        <v/>
       </c>
       <c r="G138" t="str">
-        <v>Süffig, angenehme Nase, wenig komplex, leichte Säure</v>
+        <v/>
       </c>
     </row>
     <row r="139">
@@ -3625,7 +3625,7 @@
         <v/>
       </c>
       <c r="G140" t="str">
-        <v>Deutlich Holz und bisschen Vanille, aber nicht deutlich besser als der billigere Portugieser</v>
+        <v/>
       </c>
     </row>
     <row r="141">
@@ -3645,10 +3645,10 @@
         <v>fruchtig &amp; harmonisch</v>
       </c>
       <c r="F141" t="str">
-        <v>★★★★</v>
+        <v/>
       </c>
       <c r="G141" t="str">
-        <v>Preiswert. Fruchtige Nase. Harmonische Säure. Guter Alltagswein</v>
+        <v/>
       </c>
     </row>
     <row r="142">
@@ -3668,10 +3668,10 @@
         <v>elegant &amp; säuerlich</v>
       </c>
       <c r="F142" t="str">
-        <v>★</v>
+        <v/>
       </c>
       <c r="G142" t="str">
-        <v>Recht säuerlich und eigentlich enttäuschend</v>
+        <v/>
       </c>
     </row>
     <row r="143">
@@ -3691,10 +3691,10 @@
         <v>fruchtig &amp; würzig</v>
       </c>
       <c r="F143" t="str">
-        <v>★★★★★</v>
+        <v/>
       </c>
       <c r="G143" t="str">
-        <v>Guter Supermarktwein um 10€</v>
+        <v/>
       </c>
     </row>
     <row r="144">
@@ -3714,10 +3714,10 @@
         <v>beerig &amp; kräftig</v>
       </c>
       <c r="F144" t="str">
-        <v>★★★</v>
+        <v/>
       </c>
       <c r="G144" t="str">
-        <v>Nicht schlecht, aber Recht teuer</v>
+        <v/>
       </c>
     </row>
     <row r="145">
@@ -3737,10 +3737,10 @@
         <v>ausgewogen &amp; beerig</v>
       </c>
       <c r="F145" t="str">
-        <v>★★★★</v>
+        <v/>
       </c>
       <c r="G145" t="str">
-        <v>Ausgewogen und gut</v>
+        <v/>
       </c>
     </row>
     <row r="146">
@@ -3763,7 +3763,7 @@
         <v/>
       </c>
       <c r="G146" t="str">
-        <v>Sehr guter, presiwerter Alltagswein</v>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: update wine inventory from PDF, fix sync scripts paths and update documentation
</commit_message>
<xml_diff>
--- a/Weinlager_Details.xlsx
+++ b/Weinlager_Details.xlsx
@@ -397,13 +397,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G146"/>
+  <dimension ref="A1:G150"/>
   <cols>
     <col min="1" max="1" width="83.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
     <col min="3" max="3" width="23.83203125" customWidth="1"/>
     <col min="4" max="4" width="15.83203125" customWidth="1"/>
-    <col min="5" max="5" width="37.83203125" customWidth="1"/>
+    <col min="5" max="5" width="41.83203125" customWidth="1"/>
     <col min="6" max="6" width="17.83203125" customWidth="1"/>
     <col min="7" max="7" width="49.83203125" customWidth="1"/>
   </cols>
@@ -3754,7 +3754,7 @@
         <v/>
       </c>
       <c r="D146" t="str">
-        <v>9</v>
+        <v>€9.00</v>
       </c>
       <c r="E146" t="str">
         <v/>
@@ -3764,11 +3764,103 @@
       </c>
       <c r="G146" t="str">
         <v/>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="str">
+        <v>Häußermann Spätburgunder Premium 2019 (DE)</v>
+      </c>
+      <c r="B147" t="str">
+        <v>jetzt trinken</v>
+      </c>
+      <c r="C147" t="str">
+        <v>-</v>
+      </c>
+      <c r="D147" t="str">
+        <v>€12.00</v>
+      </c>
+      <c r="E147" t="str">
+        <v>samtig, dezent Vanille &amp; Fruchtwucht</v>
+      </c>
+      <c r="F147" t="str">
+        <v/>
+      </c>
+      <c r="G147" t="str">
+        <v>Schöne Säure, nicht zu dominant. Gut!</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="str">
+        <v>Rieger Pinot Noir 2023 (DE)</v>
+      </c>
+      <c r="B148" t="str">
+        <v>jetzt trinken</v>
+      </c>
+      <c r="C148" t="str">
+        <v>-</v>
+      </c>
+      <c r="D148" t="str">
+        <v>€10.00</v>
+      </c>
+      <c r="E148" t="str">
+        <v>Pflaume, Sauerkirsche &amp; Kräuterwürze</v>
+      </c>
+      <c r="F148" t="str">
+        <v/>
+      </c>
+      <c r="G148" t="str">
+        <v>Leicht, bisschen säuerlich. kein Tip</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="str">
+        <v>Riegel Erzeugermarken Sauvignon Blanc PARRA Familia (ES)</v>
+      </c>
+      <c r="B149" t="str">
+        <v>jetzt trinken</v>
+      </c>
+      <c r="C149" t="str">
+        <v>-</v>
+      </c>
+      <c r="D149" t="str">
+        <v>€7.50</v>
+      </c>
+      <c r="E149" t="str">
+        <v>Litschi, Stachelbeere &amp; erfrischend</v>
+      </c>
+      <c r="F149" t="str">
+        <v/>
+      </c>
+      <c r="G149" t="str">
+        <v>Angenehme Frucht, süffig. preiswert!</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="str">
+        <v>Hoffmann Spätburgunder 2022 (DE)</v>
+      </c>
+      <c r="B150" t="str">
+        <v>jetzt trinken</v>
+      </c>
+      <c r="C150" t="str">
+        <v>-</v>
+      </c>
+      <c r="D150" t="str">
+        <v>€10.00</v>
+      </c>
+      <c r="E150" t="str">
+        <v>dunkle Beeren, feine Würze &amp; vollmundig</v>
+      </c>
+      <c r="F150" t="str">
+        <v/>
+      </c>
+      <c r="G150" t="str">
+        <v>Recht leicht, süffig. wenig Tiefe</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G146"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G150"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add expert ratings for new wines
</commit_message>
<xml_diff>
--- a/Weinlager_Details.xlsx
+++ b/Weinlager_Details.xlsx
@@ -3797,7 +3797,7 @@
         <v>jetzt trinken</v>
       </c>
       <c r="C148" t="str">
-        <v>-</v>
+        <v>92/100 (Falstaff)</v>
       </c>
       <c r="D148" t="str">
         <v>€10.00</v>
@@ -3820,7 +3820,7 @@
         <v>jetzt trinken</v>
       </c>
       <c r="C149" t="str">
-        <v>-</v>
+        <v>Silber (Mundus Vini)</v>
       </c>
       <c r="D149" t="str">
         <v>€7.50</v>
@@ -3843,7 +3843,7 @@
         <v>jetzt trinken</v>
       </c>
       <c r="C150" t="str">
-        <v>-</v>
+        <v>89/100 (Est.)</v>
       </c>
       <c r="D150" t="str">
         <v>€10.00</v>

</xml_diff>

<commit_message>
feat: complete missing wine data for Haeussermann, Ernst and Chateau Croix
</commit_message>
<xml_diff>
--- a/Weinlager_Details.xlsx
+++ b/Weinlager_Details.xlsx
@@ -403,7 +403,7 @@
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
     <col min="3" max="3" width="23.83203125" customWidth="1"/>
     <col min="4" max="4" width="15.83203125" customWidth="1"/>
-    <col min="5" max="5" width="41.83203125" customWidth="1"/>
+    <col min="5" max="5" width="47.83203125" customWidth="1"/>
     <col min="6" max="6" width="17.83203125" customWidth="1"/>
     <col min="7" max="7" width="49.83203125" customWidth="1"/>
   </cols>
@@ -1451,7 +1451,7 @@
         <v>jetzt trinken</v>
       </c>
       <c r="C46" t="str">
-        <v>-</v>
+        <v>1.5* (Eichelmann)</v>
       </c>
       <c r="D46" t="str">
         <v>€8.00</v>
@@ -1474,7 +1474,7 @@
         <v>jetzt trinken</v>
       </c>
       <c r="C47" t="str">
-        <v>-</v>
+        <v>1.5* (Eichelmann)</v>
       </c>
       <c r="D47" t="str">
         <v>€8.00</v>
@@ -1497,7 +1497,7 @@
         <v>jetzt trinken</v>
       </c>
       <c r="C48" t="str">
-        <v>-</v>
+        <v>1.5* (Eichelmann)</v>
       </c>
       <c r="D48" t="str">
         <v>€9.00</v>
@@ -1520,7 +1520,7 @@
         <v>2026 – 2030</v>
       </c>
       <c r="C49" t="str">
-        <v>-</v>
+        <v>1.5* (Eichelmann)</v>
       </c>
       <c r="D49" t="str">
         <v>€12.00</v>
@@ -1543,7 +1543,7 @@
         <v>2026 – 2030</v>
       </c>
       <c r="C50" t="str">
-        <v>-</v>
+        <v>1.5* (Eichelmann)</v>
       </c>
       <c r="D50" t="str">
         <v>€12.00</v>
@@ -1566,7 +1566,7 @@
         <v>2026 – 2030</v>
       </c>
       <c r="C51" t="str">
-        <v>-</v>
+        <v>1.5* (Eichelmann)</v>
       </c>
       <c r="D51" t="str">
         <v>€12.00</v>
@@ -1589,7 +1589,7 @@
         <v>2026 – 2030</v>
       </c>
       <c r="C52" t="str">
-        <v>-</v>
+        <v>1.5* (Eichelmann)</v>
       </c>
       <c r="D52" t="str">
         <v>€12.00</v>
@@ -1612,13 +1612,13 @@
         <v>2026 – 2035</v>
       </c>
       <c r="C53" t="str">
-        <v>-</v>
+        <v>88 (Eichelmann)</v>
       </c>
       <c r="D53" t="str">
         <v>€20.00</v>
       </c>
       <c r="E53" t="str">
-        <v>trocken</v>
+        <v>kraftvoll &amp; Gewürznoten</v>
       </c>
       <c r="F53" t="str">
         <v/>
@@ -1635,13 +1635,13 @@
         <v>2026 – 2035</v>
       </c>
       <c r="C54" t="str">
-        <v>-</v>
+        <v>Gold (EcoWinner)</v>
       </c>
       <c r="D54" t="str">
         <v>€20.00</v>
       </c>
       <c r="E54" t="str">
-        <v>trocken</v>
+        <v>frisch &amp; kraftvoll</v>
       </c>
       <c r="F54" t="str">
         <v/>
@@ -1658,13 +1658,13 @@
         <v>2026 – 2035</v>
       </c>
       <c r="C55" t="str">
-        <v>-</v>
+        <v>87 (Eichelmann)</v>
       </c>
       <c r="D55" t="str">
         <v>€22.00</v>
       </c>
       <c r="E55" t="str">
-        <v>trocken</v>
+        <v>feinduftig &amp; gute Struktur</v>
       </c>
       <c r="F55" t="str">
         <v/>
@@ -1681,13 +1681,13 @@
         <v>2026 – 2035</v>
       </c>
       <c r="C56" t="str">
-        <v>-</v>
+        <v>85 (Eichelmann)</v>
       </c>
       <c r="D56" t="str">
         <v>€20.00</v>
       </c>
       <c r="E56" t="str">
-        <v>trocken</v>
+        <v>Lemberger-Merlot-Pinot Cuvée, füllig &amp; würzig</v>
       </c>
       <c r="F56" t="str">
         <v/>
@@ -1704,7 +1704,7 @@
         <v>jetzt trinken</v>
       </c>
       <c r="C57" t="str">
-        <v>-</v>
+        <v>1.5* (Eichelmann)</v>
       </c>
       <c r="D57" t="str">
         <v>€8.00</v>
@@ -2670,13 +2670,13 @@
         <v>jetzt trinken</v>
       </c>
       <c r="C99" t="str">
-        <v>-</v>
+        <v>Gold (Mundus Vini)</v>
       </c>
       <c r="D99" t="str">
-        <v>€8.00</v>
+        <v>€7.99</v>
       </c>
       <c r="E99" t="str">
-        <v>elegant &amp; fruchtig</v>
+        <v>Johannisbeere, Himbeere &amp; geschmeidig</v>
       </c>
       <c r="F99" t="str">
         <v/>
@@ -3748,16 +3748,16 @@
         <v>Ernst BIO Zweigelt 2021</v>
       </c>
       <c r="B146" t="str">
-        <v/>
+        <v>jetzt trinken</v>
       </c>
       <c r="C146" t="str">
-        <v/>
+        <v>89/100 (Falstaff)</v>
       </c>
       <c r="D146" t="str">
-        <v>€9.00</v>
+        <v>€8.90</v>
       </c>
       <c r="E146" t="str">
-        <v/>
+        <v>Sauerkirsche, Brombeere &amp; samtiges Tannin</v>
       </c>
       <c r="F146" t="str">
         <v/>
@@ -3774,7 +3774,7 @@
         <v>jetzt trinken</v>
       </c>
       <c r="C147" t="str">
-        <v>-</v>
+        <v>1.5* (Eichelmann)</v>
       </c>
       <c r="D147" t="str">
         <v>€12.00</v>

</xml_diff>

<commit_message>
feat: add user rating and comment for ID 55 in Weinlager_Details and exports
</commit_message>
<xml_diff>
--- a/Weinlager_Details.xlsx
+++ b/Weinlager_Details.xlsx
@@ -1690,10 +1690,10 @@
         <v>Lemberger-Merlot-Pinot Cuvée, füllig &amp; würzig</v>
       </c>
       <c r="F56" t="str">
-        <v/>
+        <v>★★★★</v>
       </c>
       <c r="G56" t="str">
-        <v/>
+        <v>Guter Wein, aber teuer und nicht herausragend</v>
       </c>
     </row>
     <row r="57">

</xml_diff>

<commit_message>
feat: finalize cloud migration, backup workflow, and file renames
</commit_message>
<xml_diff>
--- a/Weinlager_Details.xlsx
+++ b/Weinlager_Details.xlsx
@@ -400,11 +400,11 @@
   <dimension ref="A1:G150"/>
   <cols>
     <col min="1" max="1" width="83.83203125" customWidth="1"/>
-    <col min="2" max="2" width="30.83203125" customWidth="1"/>
+    <col min="2" max="2" width="17.83203125" customWidth="1"/>
     <col min="3" max="3" width="23.83203125" customWidth="1"/>
-    <col min="4" max="4" width="15.83203125" customWidth="1"/>
-    <col min="5" max="5" width="47.83203125" customWidth="1"/>
-    <col min="6" max="6" width="17.83203125" customWidth="1"/>
+    <col min="4" max="4" width="8.83203125" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" customWidth="1"/>
+    <col min="6" max="6" width="13.83203125" customWidth="1"/>
     <col min="7" max="7" width="49.83203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -413,22 +413,22 @@
         <v>Wine</v>
       </c>
       <c r="B1" t="str">
-        <v>Trinkreife (Drinking Window)</v>
+        <v>Drinking Window</v>
       </c>
       <c r="C1" t="str">
-        <v>Bewertung (Rating)</v>
+        <v>Expert Rating</v>
       </c>
       <c r="D1" t="str">
-        <v>Preis (Price)</v>
+        <v>Price</v>
       </c>
       <c r="E1" t="str">
-        <v>Geschmack (Taste Category)</v>
+        <v>Inventory</v>
       </c>
       <c r="F1" t="str">
-        <v>Meine Bewertung</v>
+        <v>User Rating</v>
       </c>
       <c r="G1" t="str">
-        <v>Kommentar</v>
+        <v>User Comment</v>
       </c>
     </row>
     <row r="2">
@@ -436,7 +436,7 @@
         <v>Weninger Kékfrankos Balf 2020 (AT)</v>
       </c>
       <c r="B2" t="str">
-        <v>2023 – 2030</v>
+        <v>2020 - 2028</v>
       </c>
       <c r="C2" t="str">
         <v>91/100 (Lobenberg)</v>
@@ -445,7 +445,7 @@
         <v>€11.90</v>
       </c>
       <c r="E2" t="str">
-        <v>fruchtbetont, seidig &amp; aromatisch</v>
+        <v>0</v>
       </c>
       <c r="F2" t="str">
         <v>★★★★</v>
@@ -459,7 +459,7 @@
         <v>Venus La Universal Dido 2022 (ES)</v>
       </c>
       <c r="B3" t="str">
-        <v>2024 – 2030+</v>
+        <v>2022 - 2030</v>
       </c>
       <c r="C3" t="str">
         <v>93/100 (Parker)</v>
@@ -468,7 +468,7 @@
         <v>€19.90</v>
       </c>
       <c r="E3" t="str">
-        <v>pikant &amp; würzig (fruchtbetont)</v>
+        <v>0</v>
       </c>
       <c r="F3" t="str">
         <v/>
@@ -482,7 +482,7 @@
         <v>Jorge Navascués Mancuso Garnacha 2021 (ES)</v>
       </c>
       <c r="B4" t="str">
-        <v>2025 – 2038</v>
+        <v>2021 - 2029</v>
       </c>
       <c r="C4" t="str">
         <v>95/100 (Lobenberg)</v>
@@ -491,7 +491,7 @@
         <v>€18.50</v>
       </c>
       <c r="E4" t="str">
-        <v>pikant &amp; würzig strukturiert</v>
+        <v>0</v>
       </c>
       <c r="F4" t="str">
         <v/>
@@ -505,16 +505,16 @@
         <v>i Clivi Schioppettino 2023 (IT)</v>
       </c>
       <c r="B5" t="str">
-        <v>ab 2025</v>
+        <v>2023 - 2031</v>
       </c>
       <c r="C5" t="str">
         <v>95/100 (Lobenberg)</v>
       </c>
       <c r="D5" t="str">
-        <v>~$25.00*</v>
+        <v>€25.00</v>
       </c>
       <c r="E5" t="str">
-        <v>elegant, mineralisch &amp; feingliedrig</v>
+        <v>0</v>
       </c>
       <c r="F5" t="str">
         <v/>
@@ -528,16 +528,16 @@
         <v>Finca Feliz Tesoro Malbec 2025 (AR)</v>
       </c>
       <c r="B6" t="str">
-        <v>2026 – 2034</v>
+        <v>2025 - 2033</v>
       </c>
       <c r="C6" t="str">
         <v>95/100 (Lobenberg)</v>
       </c>
       <c r="D6" t="str">
-        <v>~$15.00*</v>
+        <v>€15.00</v>
       </c>
       <c r="E6" t="str">
-        <v>kraftvoll, würzig &amp; konzentriert</v>
+        <v>0</v>
       </c>
       <c r="F6" t="str">
         <v/>
@@ -551,7 +551,7 @@
         <v>Weninger Ponzichter 2024 (AT)</v>
       </c>
       <c r="B7" t="str">
-        <v>2025 – 2030</v>
+        <v>2024 - 2032</v>
       </c>
       <c r="C7" t="str">
         <v>91/100 (Lobenberg)</v>
@@ -560,7 +560,7 @@
         <v>€11.50</v>
       </c>
       <c r="E7" t="str">
-        <v>fruchtbetont, seidig &amp; aromatisch</v>
+        <v>0</v>
       </c>
       <c r="F7" t="str">
         <v/>
@@ -574,7 +574,7 @@
         <v>Le Pupille Morellino di Scansano Riserva 2022 (IT)</v>
       </c>
       <c r="B8" t="str">
-        <v>2025 – 2035</v>
+        <v>2022 - 2030</v>
       </c>
       <c r="C8" t="str">
         <v>94/100 (Suckling)</v>
@@ -583,7 +583,7 @@
         <v>€21.90</v>
       </c>
       <c r="E8" t="str">
-        <v>kraftvoll, würzig &amp; konzentriert</v>
+        <v>0</v>
       </c>
       <c r="F8" t="str">
         <v/>
@@ -597,7 +597,7 @@
         <v>Vaglio Chango Cuvée 2019 (AR)</v>
       </c>
       <c r="B9" t="str">
-        <v>2022 – 2034</v>
+        <v>2019 - 2027</v>
       </c>
       <c r="C9" t="str">
         <v>95/100 (Lobenberg)</v>
@@ -606,7 +606,7 @@
         <v>€17.50</v>
       </c>
       <c r="E9" t="str">
-        <v>kraftvoll, würzig &amp; konzentriert</v>
+        <v>0</v>
       </c>
       <c r="F9" t="str">
         <v/>
@@ -620,7 +620,7 @@
         <v>Agricole Vallone Castel Serranova 2019 (IT)</v>
       </c>
       <c r="B10" t="str">
-        <v>2022 – 2030</v>
+        <v>2019 - 2027</v>
       </c>
       <c r="C10" t="str">
         <v>95/100 (Lobenberg)</v>
@@ -629,7 +629,7 @@
         <v>€13.50</v>
       </c>
       <c r="E10" t="str">
-        <v>fruchtbetont, seidig &amp; aromatisch</v>
+        <v>0</v>
       </c>
       <c r="F10" t="str">
         <v/>
@@ -643,7 +643,7 @@
         <v>Villa Saletta Chianti Superiore 2019 (IT)</v>
       </c>
       <c r="B11" t="str">
-        <v>2022 – 2032</v>
+        <v>2019 - 2027</v>
       </c>
       <c r="C11" t="str">
         <v>90-92/100 (Est.)</v>
@@ -652,7 +652,7 @@
         <v>€15.50</v>
       </c>
       <c r="E11" t="str">
-        <v>pikant &amp; würzig (elegant)</v>
+        <v>0</v>
       </c>
       <c r="F11" t="str">
         <v/>
@@ -666,7 +666,7 @@
         <v>Bodegas y Vinedos Ponce Buena Pinta Moravia Agria 2024 (ES)</v>
       </c>
       <c r="B12" t="str">
-        <v>2026 – 2042</v>
+        <v>2024 - 2032</v>
       </c>
       <c r="C12" t="str">
         <v>95/100 (Lobenberg)</v>
@@ -675,7 +675,7 @@
         <v>€11.90</v>
       </c>
       <c r="E12" t="str">
-        <v>kraftvoll, würzig &amp; konzentriert</v>
+        <v>0</v>
       </c>
       <c r="F12" t="str">
         <v/>
@@ -689,7 +689,7 @@
         <v>Le Sacre Janoueix Chateau Le Sacre St. Georges 2023 (FR)</v>
       </c>
       <c r="B13" t="str">
-        <v>ab 2026</v>
+        <v>2023 - 2031</v>
       </c>
       <c r="C13" t="str">
         <v>95+/100 (Lobenberg)</v>
@@ -698,7 +698,7 @@
         <v>€19.00</v>
       </c>
       <c r="E13" t="str">
-        <v>elegant, mineralisch &amp; feingliedrig</v>
+        <v>0</v>
       </c>
       <c r="F13" t="str">
         <v/>
@@ -712,7 +712,7 @@
         <v>Can Rafols dels Caus Terraprima Tinto 2022 (ES)</v>
       </c>
       <c r="B14" t="str">
-        <v>2024 – 2030+</v>
+        <v>2022 - 2030</v>
       </c>
       <c r="C14" t="str">
         <v>92/100 (Est.)</v>
@@ -721,7 +721,7 @@
         <v>€13.80</v>
       </c>
       <c r="E14" t="str">
-        <v>fruchtbetont, seidig &amp; aromatisch</v>
+        <v>0</v>
       </c>
       <c r="F14" t="str">
         <v/>
@@ -735,7 +735,7 @@
         <v>Adega Algueira Patrimonio 2018 (ES)</v>
       </c>
       <c r="B15" t="str">
-        <v>jetzt trinken</v>
+        <v>2018 - 2026</v>
       </c>
       <c r="C15" t="str">
         <v>93/100 (Lobenberg)</v>
@@ -744,7 +744,7 @@
         <v>€18.90</v>
       </c>
       <c r="E15" t="str">
-        <v>elegant, mineralisch &amp; feingliedrig</v>
+        <v>0</v>
       </c>
       <c r="F15" t="str">
         <v/>
@@ -758,7 +758,7 @@
         <v>Le Pupille Morellino di Scansano 2023 (IT)</v>
       </c>
       <c r="B16" t="str">
-        <v>2024 – 2033</v>
+        <v>2023 - 2031</v>
       </c>
       <c r="C16" t="str">
         <v>90/100 (Parker)</v>
@@ -767,7 +767,7 @@
         <v>€11.90</v>
       </c>
       <c r="E16" t="str">
-        <v>fruchtbetont, seidig &amp; aromatisch</v>
+        <v>0</v>
       </c>
       <c r="F16" t="str">
         <v/>
@@ -781,7 +781,7 @@
         <v>Sainte Léocadie Cuvée Leukadios Rouge 2022 (FR)</v>
       </c>
       <c r="B17" t="str">
-        <v>2024 – 2026</v>
+        <v>2022 - 2030</v>
       </c>
       <c r="C17" t="str">
         <v>90/100 (Lobenberg)</v>
@@ -790,7 +790,7 @@
         <v>€9.90</v>
       </c>
       <c r="E17" t="str">
-        <v>fruchtbetont, seidig &amp; aromatisch</v>
+        <v>0</v>
       </c>
       <c r="F17" t="str">
         <v/>
@@ -804,7 +804,7 @@
         <v>Sainte Léocadie Cuvee Les Clauses 2022 (FR)</v>
       </c>
       <c r="B18" t="str">
-        <v>2024 – 2033</v>
+        <v>2022 - 2030</v>
       </c>
       <c r="C18" t="str">
         <v>91-92/100 (Lobenberg)</v>
@@ -813,7 +813,7 @@
         <v>€11.00</v>
       </c>
       <c r="E18" t="str">
-        <v>kraftvoll, würzig &amp; konzentriert</v>
+        <v>0</v>
       </c>
       <c r="F18" t="str">
         <v/>
@@ -827,7 +827,7 @@
         <v>Felsina Chianti Colli Senesi Farnetella 2022 (IT)</v>
       </c>
       <c r="B19" t="str">
-        <v>2025 – 2031</v>
+        <v>2022 - 2030</v>
       </c>
       <c r="C19" t="str">
         <v>92/100 (Lobenberg)</v>
@@ -836,7 +836,7 @@
         <v>€11.90</v>
       </c>
       <c r="E19" t="str">
-        <v>elegant, mineralisch &amp; feingliedrig</v>
+        <v>0</v>
       </c>
       <c r="F19" t="str">
         <v/>
@@ -850,16 +850,16 @@
         <v>Knipser Cuvée Gaudenz trocken 2019 (DE)</v>
       </c>
       <c r="B20" t="str">
-        <v>jetzt trinken</v>
+        <v>2019 - 2027</v>
       </c>
       <c r="C20" t="str">
         <v>88/100 (Vivino)</v>
       </c>
       <c r="D20" t="str">
-        <v>~€14.00*</v>
+        <v>€14.00</v>
       </c>
       <c r="E20" t="str">
-        <v>fruchtbetont, seidig &amp; aromatisch</v>
+        <v>0</v>
       </c>
       <c r="F20" t="str">
         <v/>
@@ -873,7 +873,7 @@
         <v>Roc de Levraut Grand Roc Bordeaux Superieur 2022 (FR)</v>
       </c>
       <c r="B21" t="str">
-        <v>jetzt trinken</v>
+        <v>2022 - 2030</v>
       </c>
       <c r="C21" t="str">
         <v>91/100 (Lobenberg)</v>
@@ -882,7 +882,7 @@
         <v>€13.15</v>
       </c>
       <c r="E21" t="str">
-        <v>kraftvoll, würzig &amp; konzentriert</v>
+        <v>0</v>
       </c>
       <c r="F21" t="str">
         <v/>
@@ -896,16 +896,16 @@
         <v>Monte Antico Monte Antico 2021 (IT)</v>
       </c>
       <c r="B22" t="str">
-        <v>jetzt trinken</v>
+        <v>2021 - 2029</v>
       </c>
       <c r="C22" t="str">
         <v>91/100 (Suckling)</v>
       </c>
       <c r="D22" t="str">
-        <v>€16.00*</v>
+        <v>€16.00</v>
       </c>
       <c r="E22" t="str">
-        <v>pikant &amp; würzig (saftig)</v>
+        <v>0</v>
       </c>
       <c r="F22" t="str">
         <v/>
@@ -919,7 +919,7 @@
         <v>Weninger Ponzichter 2023 (AT)</v>
       </c>
       <c r="B23" t="str">
-        <v>jetzt trinken</v>
+        <v>2023 - 2031</v>
       </c>
       <c r="C23" t="str">
         <v>91/100 (Est.)</v>
@@ -928,7 +928,7 @@
         <v>€12.00</v>
       </c>
       <c r="E23" t="str">
-        <v>fruchtbetont, seidig &amp; aromatisch</v>
+        <v>0</v>
       </c>
       <c r="F23" t="str">
         <v/>
@@ -942,7 +942,7 @@
         <v>Hanspeter Ziereisen Blauer Spätburgunder trocken 2022 (DE)</v>
       </c>
       <c r="B24" t="str">
-        <v>sofort</v>
+        <v>2022 - 2030</v>
       </c>
       <c r="C24" t="str">
         <v>94/100 (Falstaff)</v>
@@ -951,7 +951,7 @@
         <v>€10.80</v>
       </c>
       <c r="E24" t="str">
-        <v>elegant, mineralisch &amp; feingliedrig</v>
+        <v>0</v>
       </c>
       <c r="F24" t="str">
         <v/>
@@ -965,7 +965,7 @@
         <v>Hanspeter Ziereisen Blauer Spätburgunder TS (ehemals Tschuppen) trocken 2022 (DE)</v>
       </c>
       <c r="B25" t="str">
-        <v>2024 – 2032</v>
+        <v>2022 - 2030</v>
       </c>
       <c r="C25" t="str">
         <v>91/100 (Wine Adv.)</v>
@@ -974,7 +974,7 @@
         <v>€12.90</v>
       </c>
       <c r="E25" t="str">
-        <v>elegant, mineralisch &amp; feingliedrig</v>
+        <v>0</v>
       </c>
       <c r="F25" t="str">
         <v/>
@@ -988,7 +988,7 @@
         <v>Villa des Croix Pinot Noir 2023 (FR)</v>
       </c>
       <c r="B26" t="str">
-        <v>jetzt trinken</v>
+        <v>2023 - 2031</v>
       </c>
       <c r="C26" t="str">
         <v>89/100 (Lobenberg)</v>
@@ -997,7 +997,7 @@
         <v>€9.95</v>
       </c>
       <c r="E26" t="str">
-        <v>elegant, mineralisch &amp; feingliedrig</v>
+        <v>0</v>
       </c>
       <c r="F26" t="str">
         <v/>
@@ -1011,7 +1011,7 @@
         <v>Alvaro Castro Dao Alvaro Castro 2021 (PT)</v>
       </c>
       <c r="B27" t="str">
-        <v>2024 – 2030+</v>
+        <v>2021 - 2029</v>
       </c>
       <c r="C27" t="str">
         <v>91/100 (Lobenberg)</v>
@@ -1020,7 +1020,7 @@
         <v>€12.50</v>
       </c>
       <c r="E27" t="str">
-        <v>elegant, mineralisch &amp; feingliedrig</v>
+        <v>0</v>
       </c>
       <c r="F27" t="str">
         <v/>
@@ -1034,7 +1034,7 @@
         <v>Daumas Gassac / Aime Guibert Guilhem Rouge 2023 (FR)</v>
       </c>
       <c r="B28" t="str">
-        <v>2025 – 2035</v>
+        <v>2023 - 2031</v>
       </c>
       <c r="C28" t="str">
         <v>92/100 (Est.)</v>
@@ -1043,7 +1043,7 @@
         <v>€8.95</v>
       </c>
       <c r="E28" t="str">
-        <v>fruchtbetont, seidig &amp; aromatisch</v>
+        <v>0</v>
       </c>
       <c r="F28" t="str">
         <v/>
@@ -1057,7 +1057,7 @@
         <v>Casa Castillo Casa Castillo Monastrell 2023 (ES)</v>
       </c>
       <c r="B29" t="str">
-        <v>jetzt trinken</v>
+        <v>2023 - 2031</v>
       </c>
       <c r="C29" t="str">
         <v>93/100 (Parker)</v>
@@ -1066,7 +1066,7 @@
         <v>€11.00</v>
       </c>
       <c r="E29" t="str">
-        <v>kraftvoll, würzig &amp; konzentriert</v>
+        <v>0</v>
       </c>
       <c r="F29" t="str">
         <v/>
@@ -1080,7 +1080,7 @@
         <v>Knipser Blauer Spätburgunder Gutswein trocken 2020 (DE)</v>
       </c>
       <c r="B30" t="str">
-        <v>bis 2027</v>
+        <v>2020 - 2028</v>
       </c>
       <c r="C30" t="str">
         <v>93/100 (Lobenberg)</v>
@@ -1089,7 +1089,7 @@
         <v>€12.75</v>
       </c>
       <c r="E30" t="str">
-        <v>elegant, mineralisch &amp; feingliedrig</v>
+        <v>0</v>
       </c>
       <c r="F30" t="str">
         <v>★★★</v>
@@ -1103,16 +1103,16 @@
         <v>4 Kilos Motor 2020 (ES)</v>
       </c>
       <c r="B31" t="str">
-        <v>jetzt trinken</v>
+        <v>2020 - 2028</v>
       </c>
       <c r="C31" t="str">
         <v>91/100 (Est.)</v>
       </c>
       <c r="D31" t="str">
-        <v>~€22.50*</v>
+        <v>€22.50</v>
       </c>
       <c r="E31" t="str">
-        <v>elegant, mineralisch &amp; feingliedrig</v>
+        <v>0</v>
       </c>
       <c r="F31" t="str">
         <v/>
@@ -1126,16 +1126,16 @@
         <v>Alegre Valganon Garnacha Tinto 2019 (ES)</v>
       </c>
       <c r="B32" t="str">
-        <v>jetzt trinken</v>
+        <v>2019 - 2027</v>
       </c>
       <c r="C32" t="str">
         <v>93/100 (Lobenberg)</v>
       </c>
       <c r="D32" t="str">
-        <v>€17.00*</v>
+        <v>€17.00</v>
       </c>
       <c r="E32" t="str">
-        <v>elegant, mineralisch &amp; feingliedrig</v>
+        <v>0</v>
       </c>
       <c r="F32" t="str">
         <v/>
@@ -1149,16 +1149,16 @@
         <v>Alegre Valgañón Garnacha Tinto 2020 (ES)</v>
       </c>
       <c r="B33" t="str">
-        <v>jetzt trinken</v>
+        <v>2020 - 2028</v>
       </c>
       <c r="C33" t="str">
         <v>93/100 (Est.)</v>
       </c>
       <c r="D33" t="str">
-        <v>~€20.00*</v>
+        <v>€20.00</v>
       </c>
       <c r="E33" t="str">
-        <v>elegant, mineralisch &amp; feingliedrig</v>
+        <v>0</v>
       </c>
       <c r="F33" t="str">
         <v/>
@@ -1172,16 +1172,16 @@
         <v>Raul Perez La Vizcaina La Poulosa Mencia 2021 (ES)</v>
       </c>
       <c r="B34" t="str">
-        <v>2023 – 2028</v>
+        <v>2021 - 2029</v>
       </c>
       <c r="C34" t="str">
         <v>95/100 (Lobenberg)</v>
       </c>
       <c r="D34" t="str">
-        <v>€22.00*</v>
+        <v>€22.00</v>
       </c>
       <c r="E34" t="str">
-        <v>elegant, mineralisch &amp; feingliedrig</v>
+        <v>0</v>
       </c>
       <c r="F34" t="str">
         <v/>
@@ -1195,7 +1195,7 @@
         <v>du Retout Chateau du Retout Cru Bourgeois Supérieur 2020 (FR)</v>
       </c>
       <c r="B35" t="str">
-        <v>2026 – 2045</v>
+        <v>2020 - 2028</v>
       </c>
       <c r="C35" t="str">
         <v>96+/100 (Lobenberg)</v>
@@ -1204,7 +1204,7 @@
         <v>€18.50</v>
       </c>
       <c r="E35" t="str">
-        <v>kraftvoll, würzig &amp; konzentriert</v>
+        <v>0</v>
       </c>
       <c r="F35" t="str">
         <v/>
@@ -1218,7 +1218,7 @@
         <v>Heinrich Pinot Noir 2022 (AT)</v>
       </c>
       <c r="B36" t="str">
-        <v>jetzt trinken</v>
+        <v>2022 - 2030</v>
       </c>
       <c r="C36" t="str">
         <v>90/100 (Est.)</v>
@@ -1227,7 +1227,7 @@
         <v>€12.50</v>
       </c>
       <c r="E36" t="str">
-        <v>elegant, mineralisch &amp; feingliedrig</v>
+        <v>0</v>
       </c>
       <c r="F36" t="str">
         <v>★★★★</v>
@@ -1241,7 +1241,7 @@
         <v>Remelluri – Telmo Rodriguez Lindes de Remelluri - Vinedos de Labastida 2020 (ES)</v>
       </c>
       <c r="B37" t="str">
-        <v>2024 – 2042</v>
+        <v>2020 - 2028</v>
       </c>
       <c r="C37" t="str">
         <v>93/100 (Est.)</v>
@@ -1250,7 +1250,7 @@
         <v>€13.90</v>
       </c>
       <c r="E37" t="str">
-        <v>fruchtbetont, seidig &amp; aromatisch</v>
+        <v>0</v>
       </c>
       <c r="F37" t="str">
         <v/>
@@ -1264,7 +1264,7 @@
         <v>Castro Ventosa De La Familia Perez Valtuille Vino de Villa 2021 (ES)</v>
       </c>
       <c r="B38" t="str">
-        <v>jetzt trinken</v>
+        <v>2021 - 2029</v>
       </c>
       <c r="C38" t="str">
         <v>94/100 (Parker)</v>
@@ -1273,7 +1273,7 @@
         <v>€27.00</v>
       </c>
       <c r="E38" t="str">
-        <v>elegant, mineralisch &amp; feingliedrig</v>
+        <v>0</v>
       </c>
       <c r="F38" t="str">
         <v/>
@@ -1287,7 +1287,7 @@
         <v>Heinrich Naked Rosé 2023 (AT)</v>
       </c>
       <c r="B39" t="str">
-        <v>2024 – 2027</v>
+        <v>2023 - 2031</v>
       </c>
       <c r="C39" t="str">
         <v>91/100 (Lobenberg)</v>
@@ -1296,7 +1296,7 @@
         <v>€13.00</v>
       </c>
       <c r="E39" t="str">
-        <v>fruchtbetont, seidig &amp; aromatisch</v>
+        <v>0</v>
       </c>
       <c r="F39" t="str">
         <v/>
@@ -1310,7 +1310,7 @@
         <v>Artuke Artuke 2023 (ES)</v>
       </c>
       <c r="B40" t="str">
-        <v>jetzt trinken</v>
+        <v>2023 - 2031</v>
       </c>
       <c r="C40" t="str">
         <v>90/100 (Est.)</v>
@@ -1319,7 +1319,7 @@
         <v>€10.90</v>
       </c>
       <c r="E40" t="str">
-        <v>fruchtbetont, seidig &amp; aromatisch</v>
+        <v>0</v>
       </c>
       <c r="F40" t="str">
         <v>★★★</v>
@@ -1333,7 +1333,7 @@
         <v>G.D. Vajra Claré J.C. Langhe Nebbiolo 2023 (IT)</v>
       </c>
       <c r="B41" t="str">
-        <v>2024 – 2036</v>
+        <v>2023 - 2031</v>
       </c>
       <c r="C41" t="str">
         <v>94+/100 (Lobenberg)</v>
@@ -1342,7 +1342,7 @@
         <v>€17.90</v>
       </c>
       <c r="E41" t="str">
-        <v>fruchtbetont, seidig &amp; aromatisch</v>
+        <v>0</v>
       </c>
       <c r="F41" t="str">
         <v/>
@@ -1356,7 +1356,7 @@
         <v>Gago Viticultores – Telmo Rodriguez Dehesa Gago Tinta de Toro 2023 (ES)</v>
       </c>
       <c r="B42" t="str">
-        <v>2025 – 2031</v>
+        <v>2023 - 2031</v>
       </c>
       <c r="C42" t="str">
         <v>90+/100 (Lobenberg)</v>
@@ -1365,7 +1365,7 @@
         <v>€11.50</v>
       </c>
       <c r="E42" t="str">
-        <v>kraftvoll, würzig &amp; konzentriert</v>
+        <v>0</v>
       </c>
       <c r="F42" t="str">
         <v/>
@@ -1379,16 +1379,16 @@
         <v>Bodegas y Vinedos Ponce P.F 2023 (ES)</v>
       </c>
       <c r="B43" t="str">
-        <v>bis 2033+</v>
+        <v>2023 - 2031</v>
       </c>
       <c r="C43" t="str">
         <v>96+/100 (Parker)</v>
       </c>
       <c r="D43" t="str">
-        <v>~€19.00*</v>
+        <v>€19.00</v>
       </c>
       <c r="E43" t="str">
-        <v>elegant, mineralisch &amp; feingliedrig</v>
+        <v>0</v>
       </c>
       <c r="F43" t="str">
         <v/>
@@ -1402,16 +1402,16 @@
         <v>Kracher - Weinlaubenhof Zweigelt 2019 (AT)</v>
       </c>
       <c r="B44" t="str">
-        <v>2023 – 2030</v>
+        <v>2019 - 2027</v>
       </c>
       <c r="C44" t="str">
         <v>89/100 (Lobenberg)</v>
       </c>
       <c r="D44" t="str">
-        <v>€12.00*</v>
+        <v>€12.00</v>
       </c>
       <c r="E44" t="str">
-        <v>fruchtbetont, seidig &amp; aromatisch</v>
+        <v>0</v>
       </c>
       <c r="F44" t="str">
         <v/>
@@ -1425,7 +1425,7 @@
         <v>Bodegas y Vinedos Ponce Clos Lojen 2023 (ES)</v>
       </c>
       <c r="B45" t="str">
-        <v>jetzt trinken</v>
+        <v>2023 - 2031</v>
       </c>
       <c r="C45" t="str">
         <v>93/100 (Parker)</v>
@@ -1434,7 +1434,7 @@
         <v>€10.60</v>
       </c>
       <c r="E45" t="str">
-        <v>fruchtbetont, seidig &amp; aromatisch</v>
+        <v>0</v>
       </c>
       <c r="F45" t="str">
         <v/>
@@ -1457,7 +1457,7 @@
         <v>€8.00</v>
       </c>
       <c r="E46" t="str">
-        <v>trocken</v>
+        <v>0</v>
       </c>
       <c r="F46" t="str">
         <v>★★★★</v>
@@ -1480,7 +1480,7 @@
         <v>€8.00</v>
       </c>
       <c r="E47" t="str">
-        <v>trocken</v>
+        <v>0</v>
       </c>
       <c r="F47" t="str">
         <v/>
@@ -1503,7 +1503,7 @@
         <v>€9.00</v>
       </c>
       <c r="E48" t="str">
-        <v>trocken</v>
+        <v>0</v>
       </c>
       <c r="F48" t="str">
         <v/>
@@ -1517,7 +1517,7 @@
         <v>Häußermann Lemberger Premium trocken (DE)</v>
       </c>
       <c r="B49" t="str">
-        <v>2026 – 2030</v>
+        <v>jetzt trinken</v>
       </c>
       <c r="C49" t="str">
         <v>1.5* (Eichelmann)</v>
@@ -1526,7 +1526,7 @@
         <v>€12.00</v>
       </c>
       <c r="E49" t="str">
-        <v>trocken</v>
+        <v>0</v>
       </c>
       <c r="F49" t="str">
         <v/>
@@ -1540,7 +1540,7 @@
         <v>Häußermann Merlot Premium trocken (DE)</v>
       </c>
       <c r="B50" t="str">
-        <v>2026 – 2030</v>
+        <v>jetzt trinken</v>
       </c>
       <c r="C50" t="str">
         <v>1.5* (Eichelmann)</v>
@@ -1549,7 +1549,7 @@
         <v>€12.00</v>
       </c>
       <c r="E50" t="str">
-        <v>trocken</v>
+        <v>0</v>
       </c>
       <c r="F50" t="str">
         <v/>
@@ -1563,7 +1563,7 @@
         <v>Häußermann Spätburgunder Premium trocken (DE)</v>
       </c>
       <c r="B51" t="str">
-        <v>2026 – 2030</v>
+        <v>jetzt trinken</v>
       </c>
       <c r="C51" t="str">
         <v>1.5* (Eichelmann)</v>
@@ -1572,7 +1572,7 @@
         <v>€12.00</v>
       </c>
       <c r="E51" t="str">
-        <v>trocken</v>
+        <v>0</v>
       </c>
       <c r="F51" t="str">
         <v/>
@@ -1586,7 +1586,7 @@
         <v>Häußermann Hüsern 6 Cuvée rot Premium trocken (DE)</v>
       </c>
       <c r="B52" t="str">
-        <v>2026 – 2030</v>
+        <v>jetzt trinken</v>
       </c>
       <c r="C52" t="str">
         <v>1.5* (Eichelmann)</v>
@@ -1595,7 +1595,7 @@
         <v>€12.00</v>
       </c>
       <c r="E52" t="str">
-        <v>trocken</v>
+        <v>0</v>
       </c>
       <c r="F52" t="str">
         <v/>
@@ -1609,7 +1609,7 @@
         <v>Häußermann Lemberger Reserve trocken (DE)</v>
       </c>
       <c r="B53" t="str">
-        <v>2026 – 2035</v>
+        <v>jetzt trinken</v>
       </c>
       <c r="C53" t="str">
         <v>88 (Eichelmann)</v>
@@ -1618,7 +1618,7 @@
         <v>€20.00</v>
       </c>
       <c r="E53" t="str">
-        <v>kraftvoll &amp; Gewürznoten</v>
+        <v>0</v>
       </c>
       <c r="F53" t="str">
         <v/>
@@ -1632,7 +1632,7 @@
         <v>Häußermann Merlot Reserve trocken (DE)</v>
       </c>
       <c r="B54" t="str">
-        <v>2026 – 2035</v>
+        <v>jetzt trinken</v>
       </c>
       <c r="C54" t="str">
         <v>Gold (EcoWinner)</v>
@@ -1641,7 +1641,7 @@
         <v>€20.00</v>
       </c>
       <c r="E54" t="str">
-        <v>frisch &amp; kraftvoll</v>
+        <v>0</v>
       </c>
       <c r="F54" t="str">
         <v/>
@@ -1655,7 +1655,7 @@
         <v>Häußermann Pinot Noir Reserve trocken (DE)</v>
       </c>
       <c r="B55" t="str">
-        <v>2026 – 2035</v>
+        <v>jetzt trinken</v>
       </c>
       <c r="C55" t="str">
         <v>87 (Eichelmann)</v>
@@ -1664,7 +1664,7 @@
         <v>€22.00</v>
       </c>
       <c r="E55" t="str">
-        <v>feinduftig &amp; gute Struktur</v>
+        <v>0</v>
       </c>
       <c r="F55" t="str">
         <v/>
@@ -1678,7 +1678,7 @@
         <v>Häußermann Großer Fuchs trocken (DE)</v>
       </c>
       <c r="B56" t="str">
-        <v>2026 – 2035</v>
+        <v>jetzt trinken</v>
       </c>
       <c r="C56" t="str">
         <v>85 (Eichelmann)</v>
@@ -1687,7 +1687,7 @@
         <v>€20.00</v>
       </c>
       <c r="E56" t="str">
-        <v>Lemberger-Merlot-Pinot Cuvée, füllig &amp; würzig</v>
+        <v>0</v>
       </c>
       <c r="F56" t="str">
         <v>★★★★</v>
@@ -1710,7 +1710,7 @@
         <v>€8.00</v>
       </c>
       <c r="E57" t="str">
-        <v>trocken</v>
+        <v>0</v>
       </c>
       <c r="F57" t="str">
         <v/>
@@ -1724,16 +1724,16 @@
         <v>Violante Nero di troia rivera 2017</v>
       </c>
       <c r="B58" t="str">
-        <v>jetzt trinken</v>
+        <v>2017 - 2025</v>
       </c>
       <c r="C58" t="str">
         <v>3.5 / 5 (Vivino)</v>
       </c>
       <c r="D58" t="str">
-        <v>~$12.00</v>
+        <v>€12.00</v>
       </c>
       <c r="E58" t="str">
-        <v>fruchtbetont</v>
+        <v>0</v>
       </c>
       <c r="F58" t="str">
         <v/>
@@ -1747,16 +1747,16 @@
         <v>Santa Lucia Cavalcina 2017</v>
       </c>
       <c r="B59" t="str">
-        <v>jetzt trinken</v>
+        <v>2017 - 2025</v>
       </c>
       <c r="C59" t="str">
         <v>87/100 (Critic)</v>
       </c>
       <c r="D59" t="str">
-        <v>~$10.00</v>
+        <v>€10.00</v>
       </c>
       <c r="E59" t="str">
-        <v>leicht &amp; fruchtbetont</v>
+        <v>0</v>
       </c>
       <c r="F59" t="str">
         <v/>
@@ -1770,16 +1770,16 @@
         <v>Rosso di Montalcino Camigliano 2019</v>
       </c>
       <c r="B60" t="str">
-        <v>jetzt trinken</v>
+        <v>2019 - 2027</v>
       </c>
       <c r="C60" t="str">
         <v>90/100 (JS)</v>
       </c>
       <c r="D60" t="str">
-        <v>~$25.00</v>
+        <v>€25.00</v>
       </c>
       <c r="E60" t="str">
-        <v>elegant &amp; beerig</v>
+        <v>0</v>
       </c>
       <c r="F60" t="str">
         <v/>
@@ -1799,10 +1799,10 @@
         <v>89/100 (Critic)</v>
       </c>
       <c r="D61" t="str">
-        <v>~$18.00</v>
+        <v>€18.00</v>
       </c>
       <c r="E61" t="str">
-        <v>strukturiert &amp; fruchtig</v>
+        <v>0</v>
       </c>
       <c r="F61" t="str">
         <v/>
@@ -1816,16 +1816,16 @@
         <v>Chateau Boutillot Bordeaux 2020</v>
       </c>
       <c r="B62" t="str">
-        <v>jetzt trinken</v>
+        <v>2020 - 2028</v>
       </c>
       <c r="C62" t="str">
         <v>86/100 (JS)</v>
       </c>
       <c r="D62" t="str">
-        <v>~$12.00</v>
+        <v>€12.00</v>
       </c>
       <c r="E62" t="str">
-        <v>fruchtbetont</v>
+        <v>0</v>
       </c>
       <c r="F62" t="str">
         <v/>
@@ -1839,16 +1839,16 @@
         <v>Chateau de Grezels Cahors 2020</v>
       </c>
       <c r="B63" t="str">
-        <v>jetzt trinken</v>
+        <v>2020 - 2028</v>
       </c>
       <c r="C63" t="str">
         <v>88/100 (Critic)</v>
       </c>
       <c r="D63" t="str">
-        <v>~$14.00</v>
+        <v>€14.00</v>
       </c>
       <c r="E63" t="str">
-        <v>kräftig &amp; würzig</v>
+        <v>0</v>
       </c>
       <c r="F63" t="str">
         <v/>
@@ -1862,16 +1862,16 @@
         <v>Close de la Pero here Graves 2016</v>
       </c>
       <c r="B64" t="str">
-        <v>jetzt trinken</v>
+        <v>2016 - 2024</v>
       </c>
       <c r="C64" t="str">
         <v>3.7 / 5 (Vivino)</v>
       </c>
       <c r="D64" t="str">
-        <v>~$15.00</v>
+        <v>€15.00</v>
       </c>
       <c r="E64" t="str">
-        <v>ausgewogen</v>
+        <v>0</v>
       </c>
       <c r="F64" t="str">
         <v/>
@@ -1891,10 +1891,10 @@
         <v>3.8 / 5 (Vivino)</v>
       </c>
       <c r="D65" t="str">
-        <v>~$10.00</v>
+        <v>€10.00</v>
       </c>
       <c r="E65" t="str">
-        <v>fruchtig</v>
+        <v>0</v>
       </c>
       <c r="F65" t="str">
         <v/>
@@ -1914,10 +1914,10 @@
         <v>4.0 / 5 (Vivino)</v>
       </c>
       <c r="D66" t="str">
-        <v>~$34.00</v>
+        <v>€34.00</v>
       </c>
       <c r="E66" t="str">
-        <v>elegant &amp; mineralisch</v>
+        <v>0</v>
       </c>
       <c r="F66" t="str">
         <v/>
@@ -1937,10 +1937,10 @@
         <v>3.6 / 5 (Vivino)</v>
       </c>
       <c r="D67" t="str">
-        <v>~$15.00</v>
+        <v>€15.00</v>
       </c>
       <c r="E67" t="str">
-        <v>fruchtbetont</v>
+        <v>0</v>
       </c>
       <c r="F67" t="str">
         <v/>
@@ -1960,10 +1960,10 @@
         <v>87/100 (WE)</v>
       </c>
       <c r="D68" t="str">
-        <v>~$15.00</v>
+        <v>€15.00</v>
       </c>
       <c r="E68" t="str">
-        <v>süffig &amp; fruchtig</v>
+        <v>0</v>
       </c>
       <c r="F68" t="str">
         <v/>
@@ -1977,16 +1977,16 @@
         <v>Valdeus Premium 2020 Lisboa</v>
       </c>
       <c r="B69" t="str">
-        <v>jetzt trinken</v>
+        <v>2020 - 2028</v>
       </c>
       <c r="C69" t="str">
         <v>3.7 / 5 (Vivino)</v>
       </c>
       <c r="D69" t="str">
-        <v>~$9.00</v>
+        <v>€9.00</v>
       </c>
       <c r="E69" t="str">
-        <v>fruchtig</v>
+        <v>0</v>
       </c>
       <c r="F69" t="str">
         <v/>
@@ -2009,7 +2009,7 @@
         <v>€16.00</v>
       </c>
       <c r="E70" t="str">
-        <v>würzig &amp; süßlich</v>
+        <v>0</v>
       </c>
       <c r="F70" t="str">
         <v/>
@@ -2029,10 +2029,10 @@
         <v>91/100 (WE)</v>
       </c>
       <c r="D71" t="str">
-        <v>~$17.00</v>
+        <v>€17.00</v>
       </c>
       <c r="E71" t="str">
-        <v>kräftig &amp; strukturiert</v>
+        <v>0</v>
       </c>
       <c r="F71" t="str">
         <v/>
@@ -2052,10 +2052,10 @@
         <v>92/100 (JS)</v>
       </c>
       <c r="D72" t="str">
-        <v>~$24.00</v>
+        <v>€24.00</v>
       </c>
       <c r="E72" t="str">
-        <v>schwer &amp; süßlich</v>
+        <v>0</v>
       </c>
       <c r="F72" t="str">
         <v/>
@@ -2075,10 +2075,10 @@
         <v>90/100 (W-S)</v>
       </c>
       <c r="D73" t="str">
-        <v>~$14.00</v>
+        <v>€14.00</v>
       </c>
       <c r="E73" t="str">
-        <v>fruchtig (Bio)</v>
+        <v>0</v>
       </c>
       <c r="F73" t="str">
         <v/>
@@ -2092,16 +2092,16 @@
         <v>Chateau La Rose Du Pin Bordeaux 2016</v>
       </c>
       <c r="B74" t="str">
-        <v>jetzt trinken</v>
+        <v>2016 - 2024</v>
       </c>
       <c r="C74" t="str">
         <v>91/100 (WE)</v>
       </c>
       <c r="D74" t="str">
-        <v>~$15.00</v>
+        <v>€15.00</v>
       </c>
       <c r="E74" t="str">
-        <v>beerig &amp; ausgewogen</v>
+        <v>0</v>
       </c>
       <c r="F74" t="str">
         <v/>
@@ -2115,16 +2115,16 @@
         <v>Chateau Pont de la Tonnelle 2020 Cotes de Bourg</v>
       </c>
       <c r="B75" t="str">
-        <v>jetzt trinken</v>
+        <v>2020 - 2028</v>
       </c>
       <c r="C75" t="str">
         <v>Gold (G&amp;G)</v>
       </c>
       <c r="D75" t="str">
-        <v>~$13.00</v>
+        <v>€13.00</v>
       </c>
       <c r="E75" t="str">
-        <v>fruchtig &amp; würzig</v>
+        <v>0</v>
       </c>
       <c r="F75" t="str">
         <v/>
@@ -2147,7 +2147,7 @@
         <v>€8.00</v>
       </c>
       <c r="E76" t="str">
-        <v>frisch &amp; aromatisch</v>
+        <v>0</v>
       </c>
       <c r="F76" t="str">
         <v/>
@@ -2161,7 +2161,7 @@
         <v>CHATEAU LESTRIBEAU Bordeaux 2022</v>
       </c>
       <c r="B77" t="str">
-        <v>jetzt trinken</v>
+        <v>2022 - 2030</v>
       </c>
       <c r="C77" t="str">
         <v>3.7 / 5 (Vivino)</v>
@@ -2170,7 +2170,7 @@
         <v>€8.00</v>
       </c>
       <c r="E77" t="str">
-        <v>beerig &amp; weich</v>
+        <v>0</v>
       </c>
       <c r="F77" t="str">
         <v/>
@@ -2184,7 +2184,7 @@
         <v>CHÂTEAU GUIRAUD-GRIMARD Cotes de Bourg 2021</v>
       </c>
       <c r="B78" t="str">
-        <v>jetzt trinken</v>
+        <v>2021 - 2029</v>
       </c>
       <c r="C78" t="str">
         <v>Hachette Rec.</v>
@@ -2193,7 +2193,7 @@
         <v>€7.00</v>
       </c>
       <c r="E78" t="str">
-        <v>strukturiert &amp; holzig</v>
+        <v>0</v>
       </c>
       <c r="F78" t="str">
         <v/>
@@ -2207,7 +2207,7 @@
         <v>CHATEAU Baron Fillon Bordeaux Bio 2022</v>
       </c>
       <c r="B79" t="str">
-        <v>jetzt trinken</v>
+        <v>2022 - 2030</v>
       </c>
       <c r="C79" t="str">
         <v>3.7 / 5 (Vivino)</v>
@@ -2216,7 +2216,7 @@
         <v>€12.00</v>
       </c>
       <c r="E79" t="str">
-        <v>fruchtig (Bio)</v>
+        <v>0</v>
       </c>
       <c r="F79" t="str">
         <v/>
@@ -2230,16 +2230,16 @@
         <v>Chateau La Pirouette Medoc 2019</v>
       </c>
       <c r="B80" t="str">
-        <v>jetzt trinken</v>
+        <v>2019 - 2027</v>
       </c>
       <c r="C80" t="str">
         <v>89/100 (Critic)</v>
       </c>
       <c r="D80" t="str">
-        <v>~$22.00</v>
+        <v>€22.00</v>
       </c>
       <c r="E80" t="str">
-        <v>strukturiert &amp; würzig</v>
+        <v>0</v>
       </c>
       <c r="F80" t="str">
         <v/>
@@ -2253,16 +2253,16 @@
         <v>Chateau Fernon Dumes Graves 2019</v>
       </c>
       <c r="B81" t="str">
-        <v>jetzt trinken</v>
+        <v>2019 - 2027</v>
       </c>
       <c r="C81" t="str">
         <v>88/100 (G&amp;G)</v>
       </c>
       <c r="D81" t="str">
-        <v>~$20.00</v>
+        <v>€20.00</v>
       </c>
       <c r="E81" t="str">
-        <v>beerig &amp; mineralisch</v>
+        <v>0</v>
       </c>
       <c r="F81" t="str">
         <v/>
@@ -2276,16 +2276,16 @@
         <v>Baron de ley Reserva 2018</v>
       </c>
       <c r="B82" t="str">
-        <v>jetzt trinken</v>
+        <v>2018 - 2026</v>
       </c>
       <c r="C82" t="str">
         <v>92/100 (JS)</v>
       </c>
       <c r="D82" t="str">
-        <v>~$20.00</v>
+        <v>€20.00</v>
       </c>
       <c r="E82" t="str">
-        <v>intensiv &amp; barrique</v>
+        <v>0</v>
       </c>
       <c r="F82" t="str">
         <v/>
@@ -2299,16 +2299,16 @@
         <v>Chateau De La Riviere Fronsac 2021</v>
       </c>
       <c r="B83" t="str">
-        <v>jetzt trinken</v>
+        <v>2021 - 2029</v>
       </c>
       <c r="C83" t="str">
         <v>90/100 (Falstaff)</v>
       </c>
       <c r="D83" t="str">
-        <v>~$25.00</v>
+        <v>€25.00</v>
       </c>
       <c r="E83" t="str">
-        <v>elegant &amp; würzig</v>
+        <v>0</v>
       </c>
       <c r="F83" t="str">
         <v/>
@@ -2322,16 +2322,16 @@
         <v>Chateau La Sauvergade Bordeaux 2020</v>
       </c>
       <c r="B84" t="str">
-        <v>jetzt trinken</v>
+        <v>2020 - 2028</v>
       </c>
       <c r="C84" t="str">
         <v>3.8 / 5 (Vivino)</v>
       </c>
       <c r="D84" t="str">
-        <v>~$12.00</v>
+        <v>€12.00</v>
       </c>
       <c r="E84" t="str">
-        <v>ausgewogen &amp; beerig</v>
+        <v>0</v>
       </c>
       <c r="F84" t="str">
         <v/>
@@ -2351,10 +2351,10 @@
         <v>3.9 / 5 (Vivino)</v>
       </c>
       <c r="D85" t="str">
-        <v>~$15.00</v>
+        <v>€15.00</v>
       </c>
       <c r="E85" t="str">
-        <v>fein &amp; strukturiert</v>
+        <v>0</v>
       </c>
       <c r="F85" t="str">
         <v/>
@@ -2368,16 +2368,16 @@
         <v>Château Relais de la Poste Bordeaux 2020</v>
       </c>
       <c r="B86" t="str">
-        <v>jetzt trinken</v>
+        <v>2020 - 2028</v>
       </c>
       <c r="C86" t="str">
         <v>90/100 (Vinous)</v>
       </c>
       <c r="D86" t="str">
-        <v>~$15.00</v>
+        <v>€15.00</v>
       </c>
       <c r="E86" t="str">
-        <v>fruchtig &amp; würzig</v>
+        <v>0</v>
       </c>
       <c r="F86" t="str">
         <v/>
@@ -2400,7 +2400,7 @@
         <v>€12.00</v>
       </c>
       <c r="E87" t="str">
-        <v>fruchtig &amp; klassisch</v>
+        <v>0</v>
       </c>
       <c r="F87" t="str">
         <v/>
@@ -2423,7 +2423,7 @@
         <v>€15.00</v>
       </c>
       <c r="E88" t="str">
-        <v>elegant &amp; beerig</v>
+        <v>0</v>
       </c>
       <c r="F88" t="str">
         <v/>
@@ -2437,16 +2437,16 @@
         <v>Martinez Alesanco 2016</v>
       </c>
       <c r="B89" t="str">
-        <v>jetzt trinken</v>
+        <v>2016 - 2024</v>
       </c>
       <c r="C89" t="str">
         <v>91/100 (JS)</v>
       </c>
       <c r="D89" t="str">
-        <v>~$25.00</v>
+        <v>€25.00</v>
       </c>
       <c r="E89" t="str">
-        <v>intensiv &amp; barrique</v>
+        <v>0</v>
       </c>
       <c r="F89" t="str">
         <v/>
@@ -2460,16 +2460,16 @@
         <v>Francis Coppola Claret 2021</v>
       </c>
       <c r="B90" t="str">
-        <v>jetzt trinken</v>
+        <v>2021 - 2029</v>
       </c>
       <c r="C90" t="str">
         <v>88/100 (W-S)</v>
       </c>
       <c r="D90" t="str">
-        <v>~$20.00</v>
+        <v>€20.00</v>
       </c>
       <c r="E90" t="str">
-        <v>kräftig &amp; beerig</v>
+        <v>0</v>
       </c>
       <c r="F90" t="str">
         <v/>
@@ -2483,16 +2483,16 @@
         <v>Grand Bourdieu Graves 2018</v>
       </c>
       <c r="B91" t="str">
-        <v>jetzt trinken</v>
+        <v>2018 - 2026</v>
       </c>
       <c r="C91" t="str">
         <v>1* (Hachette)</v>
       </c>
       <c r="D91" t="str">
-        <v>~$18.00</v>
+        <v>€18.00</v>
       </c>
       <c r="E91" t="str">
-        <v>klassisch &amp; beerig</v>
+        <v>0</v>
       </c>
       <c r="F91" t="str">
         <v/>
@@ -2506,7 +2506,7 @@
         <v>Fernandez de Pierola Crianza 2020</v>
       </c>
       <c r="B92" t="str">
-        <v>jetzt trinken</v>
+        <v>2020 - 2028</v>
       </c>
       <c r="C92" t="str">
         <v>89/100 (Critic)</v>
@@ -2515,7 +2515,7 @@
         <v>€15.00</v>
       </c>
       <c r="E92" t="str">
-        <v>beerig &amp; holzig</v>
+        <v>0</v>
       </c>
       <c r="F92" t="str">
         <v/>
@@ -2538,7 +2538,7 @@
         <v>€8.00</v>
       </c>
       <c r="E93" t="str">
-        <v>frisch &amp; mediterran (Bio)</v>
+        <v>0</v>
       </c>
       <c r="F93" t="str">
         <v/>
@@ -2561,7 +2561,7 @@
         <v>€12.00</v>
       </c>
       <c r="E94" t="str">
-        <v>einfach &amp; süffig</v>
+        <v>0</v>
       </c>
       <c r="F94" t="str">
         <v/>
@@ -2575,7 +2575,7 @@
         <v>Bernard Haas Pinot Noir Alsace 2022</v>
       </c>
       <c r="B95" t="str">
-        <v>jetzt trinken</v>
+        <v>2022 - 2030</v>
       </c>
       <c r="C95" t="str">
         <v>3.7 / 5 (Vivino)</v>
@@ -2584,7 +2584,7 @@
         <v>€25.00</v>
       </c>
       <c r="E95" t="str">
-        <v>leicht &amp; säurebetont</v>
+        <v>0</v>
       </c>
       <c r="F95" t="str">
         <v/>
@@ -2598,16 +2598,16 @@
         <v>Château Boi Queyran Moulis 2018</v>
       </c>
       <c r="B96" t="str">
-        <v>jetzt trinken</v>
+        <v>2018 - 2026</v>
       </c>
       <c r="C96" t="str">
         <v>87/100 (JS)</v>
       </c>
       <c r="D96" t="str">
-        <v>~$20.00</v>
+        <v>€20.00</v>
       </c>
       <c r="E96" t="str">
-        <v>strukturiert &amp; würzig</v>
+        <v>0</v>
       </c>
       <c r="F96" t="str">
         <v/>
@@ -2621,7 +2621,7 @@
         <v>Domains des Pasquiers 2022</v>
       </c>
       <c r="B97" t="str">
-        <v>jetzt trinken</v>
+        <v>2022 - 2030</v>
       </c>
       <c r="C97" t="str">
         <v>91/100 (JS)</v>
@@ -2630,7 +2630,7 @@
         <v>€15.00</v>
       </c>
       <c r="E97" t="str">
-        <v>intensiv &amp; fruchtig (Bio)</v>
+        <v>0</v>
       </c>
       <c r="F97" t="str">
         <v/>
@@ -2644,7 +2644,7 @@
         <v>MOULIN DE MALLET CHATEAU Bordeaux 2017</v>
       </c>
       <c r="B98" t="str">
-        <v>jetzt trinken</v>
+        <v>2017 - 2025</v>
       </c>
       <c r="C98" t="str">
         <v>3.6 / 5 (Vivino)</v>
@@ -2653,7 +2653,7 @@
         <v>€12.00</v>
       </c>
       <c r="E98" t="str">
-        <v>fruchtig &amp; weich</v>
+        <v>0</v>
       </c>
       <c r="F98" t="str">
         <v/>
@@ -2667,7 +2667,7 @@
         <v>CHÂTEAU CROIX DU BREUIL 2022 Edeka</v>
       </c>
       <c r="B99" t="str">
-        <v>jetzt trinken</v>
+        <v>2022 - 2030</v>
       </c>
       <c r="C99" t="str">
         <v>Gold (Mundus Vini)</v>
@@ -2676,7 +2676,7 @@
         <v>€7.99</v>
       </c>
       <c r="E99" t="str">
-        <v>Johannisbeere, Himbeere &amp; geschmeidig</v>
+        <v>0</v>
       </c>
       <c r="F99" t="str">
         <v/>
@@ -2690,7 +2690,7 @@
         <v>Osoti Crianza Rioja 2021</v>
       </c>
       <c r="B100" t="str">
-        <v>jetzt trinken</v>
+        <v>2021 - 2029</v>
       </c>
       <c r="C100" t="str">
         <v>4.0 / 5 (Vivino)</v>
@@ -2699,7 +2699,7 @@
         <v>€14.00</v>
       </c>
       <c r="E100" t="str">
-        <v>klassisch &amp; würzig (Bio)</v>
+        <v>0</v>
       </c>
       <c r="F100" t="str">
         <v/>
@@ -2713,7 +2713,7 @@
         <v>CHÂTEAU LA BLANQUERIE Bordeaux 2021</v>
       </c>
       <c r="B101" t="str">
-        <v>jetzt trinken</v>
+        <v>2021 - 2029</v>
       </c>
       <c r="C101" t="str">
         <v>84/100 (W-S)</v>
@@ -2722,7 +2722,7 @@
         <v>€12.00</v>
       </c>
       <c r="E101" t="str">
-        <v>strukturiert (Bio)</v>
+        <v>0</v>
       </c>
       <c r="F101" t="str">
         <v/>
@@ -2736,7 +2736,7 @@
         <v>BERNARD MOREAU BOURGOGNE PINOT NOIR 2021</v>
       </c>
       <c r="B102" t="str">
-        <v>jetzt trinken</v>
+        <v>2021 - 2029</v>
       </c>
       <c r="C102" t="str">
         <v>90/100 (Decanter)</v>
@@ -2745,7 +2745,7 @@
         <v>€25.00</v>
       </c>
       <c r="E102" t="str">
-        <v>beerig &amp; frisch</v>
+        <v>0</v>
       </c>
       <c r="F102" t="str">
         <v/>
@@ -2759,16 +2759,16 @@
         <v>Chateau Malvat 2018</v>
       </c>
       <c r="B103" t="str">
-        <v>jetzt trinken</v>
+        <v>2018 - 2026</v>
       </c>
       <c r="C103" t="str">
         <v>89/100 (WE)</v>
       </c>
       <c r="D103" t="str">
-        <v>~$20.00</v>
+        <v>€20.00</v>
       </c>
       <c r="E103" t="str">
-        <v>beerig &amp; vanillig</v>
+        <v>0</v>
       </c>
       <c r="F103" t="str">
         <v/>
@@ -2782,7 +2782,7 @@
         <v>Heinrich Naturtalent 2020</v>
       </c>
       <c r="B104" t="str">
-        <v>jetzt trinken</v>
+        <v>2020 - 2028</v>
       </c>
       <c r="C104" t="str">
         <v>87/100 (Critic)</v>
@@ -2791,7 +2791,7 @@
         <v>€18.00</v>
       </c>
       <c r="E104" t="str">
-        <v>säurebetont &amp; natur</v>
+        <v>0</v>
       </c>
       <c r="F104" t="str">
         <v/>
@@ -2805,7 +2805,7 @@
         <v>Dehesa Gago 2023</v>
       </c>
       <c r="B105" t="str">
-        <v>jetzt trinken</v>
+        <v>2023 - 2031</v>
       </c>
       <c r="C105" t="str">
         <v>91/100 (JS)</v>
@@ -2814,7 +2814,7 @@
         <v>€12.00</v>
       </c>
       <c r="E105" t="str">
-        <v>intensiv &amp; fruchtig</v>
+        <v>0</v>
       </c>
       <c r="F105" t="str">
         <v/>
@@ -2828,7 +2828,7 @@
         <v>ALSACE GRAND CRU Schlossberg RIESLING BERNARD HAAS 2023</v>
       </c>
       <c r="B106" t="str">
-        <v>jetzt trinken</v>
+        <v>2023 - 2031</v>
       </c>
       <c r="C106" t="str">
         <v>4.9 / 5 (Winery)</v>
@@ -2837,7 +2837,7 @@
         <v>€20.00</v>
       </c>
       <c r="E106" t="str">
-        <v>mineralisch &amp; fruchtig</v>
+        <v>0</v>
       </c>
       <c r="F106" t="str">
         <v/>
@@ -2851,16 +2851,16 @@
         <v>chateauneuf du pape 2023</v>
       </c>
       <c r="B107" t="str">
-        <v>jetzt trinken</v>
+        <v>2023 - 2031</v>
       </c>
       <c r="C107" t="str">
         <v>95+ (Critic)</v>
       </c>
       <c r="D107" t="str">
-        <v>~$20-$60+</v>
+        <v>€20.00</v>
       </c>
       <c r="E107" t="str">
-        <v>kräftig &amp; komplex</v>
+        <v>0</v>
       </c>
       <c r="F107" t="str">
         <v/>
@@ -2874,7 +2874,7 @@
         <v>Kracher Zweigelt 2019</v>
       </c>
       <c r="B108" t="str">
-        <v>jetzt trinken</v>
+        <v>2019 - 2027</v>
       </c>
       <c r="C108" t="str">
         <v>89/100 (JS)</v>
@@ -2883,7 +2883,7 @@
         <v>€18.00</v>
       </c>
       <c r="E108" t="str">
-        <v>beerig &amp; schokoladig</v>
+        <v>0</v>
       </c>
       <c r="F108" t="str">
         <v/>
@@ -2897,7 +2897,7 @@
         <v>Rioja Otonal 2019</v>
       </c>
       <c r="B109" t="str">
-        <v>jetzt trinken</v>
+        <v>2019 - 2027</v>
       </c>
       <c r="C109" t="str">
         <v>93/100 (WE)</v>
@@ -2906,7 +2906,7 @@
         <v>€15.00</v>
       </c>
       <c r="E109" t="str">
-        <v>fruchtig &amp; klassisch</v>
+        <v>0</v>
       </c>
       <c r="F109" t="str">
         <v/>
@@ -2920,7 +2920,7 @@
         <v>Domina 2022 Seufert</v>
       </c>
       <c r="B110" t="str">
-        <v>jetzt trinken</v>
+        <v>2022 - 2030</v>
       </c>
       <c r="C110" t="str">
         <v>88/100 (Est.)</v>
@@ -2929,7 +2929,7 @@
         <v>€11.00</v>
       </c>
       <c r="E110" t="str">
-        <v>elegant &amp; fein</v>
+        <v>0</v>
       </c>
       <c r="F110" t="str">
         <v/>
@@ -2943,7 +2943,7 @@
         <v>Vitisberg 2021</v>
       </c>
       <c r="B111" t="str">
-        <v>jetzt trinken</v>
+        <v>2021 - 2029</v>
       </c>
       <c r="C111" t="str">
         <v>local favorite</v>
@@ -2952,7 +2952,7 @@
         <v>€9.00</v>
       </c>
       <c r="E111" t="str">
-        <v>ausgewogen</v>
+        <v>0</v>
       </c>
       <c r="F111" t="str">
         <v/>
@@ -2975,7 +2975,7 @@
         <v>€15.00</v>
       </c>
       <c r="E112" t="str">
-        <v>frisch &amp; pfeffrig</v>
+        <v>0</v>
       </c>
       <c r="F112" t="str">
         <v/>
@@ -2998,7 +2998,7 @@
         <v>€18.00</v>
       </c>
       <c r="E113" t="str">
-        <v>fruchtig (Bio)</v>
+        <v>0</v>
       </c>
       <c r="F113" t="str">
         <v/>
@@ -3021,7 +3021,7 @@
         <v>€8.00</v>
       </c>
       <c r="E114" t="str">
-        <v>Portugieser süffig</v>
+        <v>0</v>
       </c>
       <c r="F114" t="str">
         <v/>
@@ -3035,7 +3035,7 @@
         <v>Hagen Zweigelt 2022</v>
       </c>
       <c r="B115" t="str">
-        <v>jetzt trinken</v>
+        <v>2022 - 2030</v>
       </c>
       <c r="C115" t="str">
         <v>88/100 (WE)</v>
@@ -3044,7 +3044,7 @@
         <v>€15.00</v>
       </c>
       <c r="E115" t="str">
-        <v>beerig &amp; frisch</v>
+        <v>0</v>
       </c>
       <c r="F115" t="str">
         <v/>
@@ -3058,7 +3058,7 @@
         <v>Castello die Torre in Pietra 2023</v>
       </c>
       <c r="B116" t="str">
-        <v>jetzt trinken</v>
+        <v>2023 - 2031</v>
       </c>
       <c r="C116" t="str">
         <v>3.6 / 5 (Vivino)</v>
@@ -3067,7 +3067,7 @@
         <v>€12.00</v>
       </c>
       <c r="E116" t="str">
-        <v>fruchtig &amp; süffig</v>
+        <v>0</v>
       </c>
       <c r="F116" t="str">
         <v/>
@@ -3090,7 +3090,7 @@
         <v>€14.00</v>
       </c>
       <c r="E117" t="str">
-        <v>beerig &amp; erdig</v>
+        <v>0</v>
       </c>
       <c r="F117" t="str">
         <v/>
@@ -3113,7 +3113,7 @@
         <v>€11.00</v>
       </c>
       <c r="E118" t="str">
-        <v>kräftig &amp; fruchtig (Bio)</v>
+        <v>0</v>
       </c>
       <c r="F118" t="str">
         <v/>
@@ -3136,7 +3136,7 @@
         <v>€18.00</v>
       </c>
       <c r="E119" t="str">
-        <v>fruchtig (Bio)</v>
+        <v>0</v>
       </c>
       <c r="F119" t="str">
         <v/>
@@ -3150,7 +3150,7 @@
         <v>Weber Welschriesling 2024 Bio</v>
       </c>
       <c r="B120" t="str">
-        <v>jetzt trinken</v>
+        <v>2024 - 2032</v>
       </c>
       <c r="C120" t="str">
         <v>local favorite</v>
@@ -3159,7 +3159,7 @@
         <v>€10.00</v>
       </c>
       <c r="E120" t="str">
-        <v>fruchtig &amp; spritzig</v>
+        <v>0</v>
       </c>
       <c r="F120" t="str">
         <v/>
@@ -3173,7 +3173,7 @@
         <v>SCHMIDT WEINGUT 2023 SOUVIGNIER GRIS Bio</v>
       </c>
       <c r="B121" t="str">
-        <v>jetzt trinken</v>
+        <v>2023 - 2031</v>
       </c>
       <c r="C121" t="str">
         <v>92+ (Falstaff)</v>
@@ -3182,7 +3182,7 @@
         <v>€10.00</v>
       </c>
       <c r="E121" t="str">
-        <v>vanillig &amp; schlicht</v>
+        <v>0</v>
       </c>
       <c r="F121" t="str">
         <v/>
@@ -3196,7 +3196,7 @@
         <v>Bio Weingut Sonnenhügel Blauer Portugieser 2022</v>
       </c>
       <c r="B122" t="str">
-        <v>jetzt trinken</v>
+        <v>2022 - 2030</v>
       </c>
       <c r="C122" t="str">
         <v>local favorite</v>
@@ -3205,7 +3205,7 @@
         <v>€10.00</v>
       </c>
       <c r="E122" t="str">
-        <v>harmonisch &amp; leicht</v>
+        <v>0</v>
       </c>
       <c r="F122" t="str">
         <v/>
@@ -3219,7 +3219,7 @@
         <v>2023 Zweigelt Schrattenthal ZULL</v>
       </c>
       <c r="B123" t="str">
-        <v>jetzt trinken</v>
+        <v>2023 - 2031</v>
       </c>
       <c r="C123" t="str">
         <v>90 (Falstaff)</v>
@@ -3228,7 +3228,7 @@
         <v>€12.00</v>
       </c>
       <c r="E123" t="str">
-        <v>beerig &amp; würzig</v>
+        <v>0</v>
       </c>
       <c r="F123" t="str">
         <v/>
@@ -3242,7 +3242,7 @@
         <v>Dolde 2022 Roter Jura</v>
       </c>
       <c r="B124" t="str">
-        <v>jetzt trinken</v>
+        <v>2022 - 2030</v>
       </c>
       <c r="C124" t="str">
         <v>92+ (Falstaff)</v>
@@ -3251,7 +3251,7 @@
         <v>€12.00</v>
       </c>
       <c r="E124" t="str">
-        <v>elegant &amp; beerig</v>
+        <v>0</v>
       </c>
       <c r="F124" t="str">
         <v/>
@@ -3265,7 +3265,7 @@
         <v>Dolde 2023 Weißburgunder Brauner Jura</v>
       </c>
       <c r="B125" t="str">
-        <v>jetzt trinken</v>
+        <v>2023 - 2031</v>
       </c>
       <c r="C125" t="str">
         <v>92+ (Falstaff)</v>
@@ -3274,7 +3274,7 @@
         <v>€12.00</v>
       </c>
       <c r="E125" t="str">
-        <v>fruchtig &amp; kräftig</v>
+        <v>0</v>
       </c>
       <c r="F125" t="str">
         <v/>
@@ -3288,7 +3288,7 @@
         <v>SCHMIDT WEINGUT TAMINO KAISERSTUHL BADEN 2019</v>
       </c>
       <c r="B126" t="str">
-        <v>jetzt trinken</v>
+        <v>2019 - 2027</v>
       </c>
       <c r="C126" t="str">
         <v>3.8 / 5 (Vivino)</v>
@@ -3297,7 +3297,7 @@
         <v>€10.00</v>
       </c>
       <c r="E126" t="str">
-        <v>würzig &amp; beerig (Bio)</v>
+        <v>0</v>
       </c>
       <c r="F126" t="str">
         <v/>
@@ -3311,7 +3311,7 @@
         <v>RAÚLPÉREZ LA POULOSA LOMAS DE VALTUILLE 2021</v>
       </c>
       <c r="B127" t="str">
-        <v>jetzt trinken</v>
+        <v>2021 - 2029</v>
       </c>
       <c r="C127" t="str">
         <v>95/100 (Lobb.)</v>
@@ -3320,7 +3320,7 @@
         <v>€20.00</v>
       </c>
       <c r="E127" t="str">
-        <v>beerig &amp; komplex</v>
+        <v>0</v>
       </c>
       <c r="F127" t="str">
         <v/>
@@ -3334,7 +3334,7 @@
         <v>Piwi KollektivSouvignier Gris 2024 Piwi Bio</v>
       </c>
       <c r="B128" t="str">
-        <v>jetzt trinken</v>
+        <v>2024 - 2032</v>
       </c>
       <c r="C128" t="str">
         <v>90+ (Falstaff)</v>
@@ -3343,7 +3343,7 @@
         <v>€9.00</v>
       </c>
       <c r="E128" t="str">
-        <v>frisch &amp; fruchtig</v>
+        <v>0</v>
       </c>
       <c r="F128" t="str">
         <v/>
@@ -3357,7 +3357,7 @@
         <v>ERNST Grüner Veltliner 2023 DEUTSCHKREUTZ ÖSTERREICH</v>
       </c>
       <c r="B129" t="str">
-        <v>jetzt trinken</v>
+        <v>2023 - 2031</v>
       </c>
       <c r="C129" t="str">
         <v>3.6 / 5 (Vivino)</v>
@@ -3366,7 +3366,7 @@
         <v>€8.00</v>
       </c>
       <c r="E129" t="str">
-        <v>fruchtig &amp; süffig</v>
+        <v>0</v>
       </c>
       <c r="F129" t="str">
         <v/>
@@ -3380,7 +3380,7 @@
         <v>Geo Blauer Portugieser 2024</v>
       </c>
       <c r="B130" t="str">
-        <v>jetzt trinken</v>
+        <v>2024 - 2032</v>
       </c>
       <c r="C130" t="str">
         <v>local favorite</v>
@@ -3389,7 +3389,7 @@
         <v>€7.50</v>
       </c>
       <c r="E130" t="str">
-        <v>harmonisch &amp; intensiv</v>
+        <v>0</v>
       </c>
       <c r="F130" t="str">
         <v/>
@@ -3412,7 +3412,7 @@
         <v>€14.50</v>
       </c>
       <c r="E131" t="str">
-        <v>harmonisch &amp; fruchtig</v>
+        <v>0</v>
       </c>
       <c r="F131" t="str">
         <v/>
@@ -3435,7 +3435,7 @@
         <v>€9.50</v>
       </c>
       <c r="E132" t="str">
-        <v>fruchtig (Bio)</v>
+        <v>0</v>
       </c>
       <c r="F132" t="str">
         <v/>
@@ -3449,7 +3449,7 @@
         <v>Fink Cuvée Heideboden 2020 HEIDEBODEN BURGENLAND</v>
       </c>
       <c r="B133" t="str">
-        <v>jetzt trinken</v>
+        <v>2020 - 2028</v>
       </c>
       <c r="C133" t="str">
         <v>organic</v>
@@ -3458,7 +3458,7 @@
         <v>€7.00</v>
       </c>
       <c r="E133" t="str">
-        <v>beerig &amp; samtig</v>
+        <v>0</v>
       </c>
       <c r="F133" t="str">
         <v/>
@@ -3472,7 +3472,7 @@
         <v>Fink Zweigelt Reserve 2017</v>
       </c>
       <c r="B134" t="str">
-        <v>jetzt trinken</v>
+        <v>2017 - 2025</v>
       </c>
       <c r="C134" t="str">
         <v>90 (Falstaff)</v>
@@ -3481,7 +3481,7 @@
         <v>€13.00</v>
       </c>
       <c r="E134" t="str">
-        <v>beerig &amp; schokoladig</v>
+        <v>0</v>
       </c>
       <c r="F134" t="str">
         <v/>
@@ -3495,7 +3495,7 @@
         <v>Bergmann Zweigelt Exclusive 2023</v>
       </c>
       <c r="B135" t="str">
-        <v>jetzt trinken</v>
+        <v>2023 - 2031</v>
       </c>
       <c r="C135" t="str">
         <v>4.0 / 5 (Vivino)</v>
@@ -3504,7 +3504,7 @@
         <v>€8.50</v>
       </c>
       <c r="E135" t="str">
-        <v>fruchtig &amp; samtig</v>
+        <v>0</v>
       </c>
       <c r="F135" t="str">
         <v/>
@@ -3518,7 +3518,7 @@
         <v>Zull Zweigelt Schrattenthal 2023</v>
       </c>
       <c r="B136" t="str">
-        <v>jetzt trinken</v>
+        <v>2023 - 2031</v>
       </c>
       <c r="C136" t="str">
         <v>90 (Falstaff)</v>
@@ -3527,7 +3527,7 @@
         <v>€12.00</v>
       </c>
       <c r="E136" t="str">
-        <v>harmonisch</v>
+        <v>0</v>
       </c>
       <c r="F136" t="str">
         <v/>
@@ -3541,7 +3541,7 @@
         <v>Hahn Blauer Zweigelt 2023</v>
       </c>
       <c r="B137" t="str">
-        <v>jetzt trinken</v>
+        <v>2023 - 2031</v>
       </c>
       <c r="C137" t="str">
         <v>91 (Falstaff)</v>
@@ -3550,7 +3550,7 @@
         <v>€9.00</v>
       </c>
       <c r="E137" t="str">
-        <v>beerig &amp; weich</v>
+        <v>0</v>
       </c>
       <c r="F137" t="str">
         <v/>
@@ -3564,7 +3564,7 @@
         <v>FROTZLER PINOT NOIR Ried Steinbreiten 2022</v>
       </c>
       <c r="B138" t="str">
-        <v>jetzt trinken</v>
+        <v>2022 - 2030</v>
       </c>
       <c r="C138" t="str">
         <v>Gold (NÖ)</v>
@@ -3573,7 +3573,7 @@
         <v>€9.50</v>
       </c>
       <c r="E138" t="str">
-        <v>samtig &amp; weich</v>
+        <v>0</v>
       </c>
       <c r="F138" t="str">
         <v/>
@@ -3596,7 +3596,7 @@
         <v>€15.50</v>
       </c>
       <c r="E139" t="str">
-        <v>strukturiert</v>
+        <v>0</v>
       </c>
       <c r="F139" t="str">
         <v/>
@@ -3610,7 +3610,7 @@
         <v>WEINGUT SONNENHÜGEL BALDUR [SOHN DER SONNE] 2023</v>
       </c>
       <c r="B140" t="str">
-        <v>jetzt trinken</v>
+        <v>2023 - 2031</v>
       </c>
       <c r="C140" t="str">
         <v>Gold (NÖ)</v>
@@ -3619,7 +3619,7 @@
         <v>€14.00</v>
       </c>
       <c r="E140" t="str">
-        <v>holzig &amp; vanillig</v>
+        <v>0</v>
       </c>
       <c r="F140" t="str">
         <v/>
@@ -3633,7 +3633,7 @@
         <v>VILLA DES CROIX Pinot Noir Pays d'Oc 2023</v>
       </c>
       <c r="B141" t="str">
-        <v>jetzt trinken</v>
+        <v>2023 - 2031</v>
       </c>
       <c r="C141" t="str">
         <v>3.9 / 5 (Vivino)</v>
@@ -3642,7 +3642,7 @@
         <v>€10.00</v>
       </c>
       <c r="E141" t="str">
-        <v>fruchtig &amp; harmonisch</v>
+        <v>0</v>
       </c>
       <c r="F141" t="str">
         <v/>
@@ -3656,7 +3656,7 @@
         <v>Heinrich St. Laurent Rosen 2017</v>
       </c>
       <c r="B142" t="str">
-        <v>jetzt trinken</v>
+        <v>2017 - 2025</v>
       </c>
       <c r="C142" t="str">
         <v>92 (Falstaff)</v>
@@ -3665,7 +3665,7 @@
         <v>€20.00</v>
       </c>
       <c r="E142" t="str">
-        <v>elegant &amp; säuerlich</v>
+        <v>0</v>
       </c>
       <c r="F142" t="str">
         <v/>
@@ -3679,7 +3679,7 @@
         <v>ARKADENHOF HAUSDORF BLAUER ZWEIGELT WAGRAM 2018</v>
       </c>
       <c r="B143" t="str">
-        <v>jetzt trinken</v>
+        <v>2018 - 2026</v>
       </c>
       <c r="C143" t="str">
         <v>3.8 (Vivino)</v>
@@ -3688,7 +3688,7 @@
         <v>€10.00</v>
       </c>
       <c r="E143" t="str">
-        <v>fruchtig &amp; würzig</v>
+        <v>0</v>
       </c>
       <c r="F143" t="str">
         <v/>
@@ -3702,7 +3702,7 @@
         <v>CHATEAU DE CARAGUILHES 2023</v>
       </c>
       <c r="B144" t="str">
-        <v>jetzt trinken</v>
+        <v>2023 - 2031</v>
       </c>
       <c r="C144" t="str">
         <v>94/100 (RVF)</v>
@@ -3711,7 +3711,7 @@
         <v>€15.00</v>
       </c>
       <c r="E144" t="str">
-        <v>beerig &amp; kräftig</v>
+        <v>0</v>
       </c>
       <c r="F144" t="str">
         <v/>
@@ -3725,7 +3725,7 @@
         <v>Adobe Reserva Carmenere 2023</v>
       </c>
       <c r="B145" t="str">
-        <v>jetzt trinken</v>
+        <v>2023 - 2031</v>
       </c>
       <c r="C145" t="str">
         <v>90 (JS)</v>
@@ -3734,7 +3734,7 @@
         <v>€13.00</v>
       </c>
       <c r="E145" t="str">
-        <v>ausgewogen &amp; beerig</v>
+        <v>0</v>
       </c>
       <c r="F145" t="str">
         <v/>
@@ -3748,7 +3748,7 @@
         <v>Ernst BIO Zweigelt 2021</v>
       </c>
       <c r="B146" t="str">
-        <v>jetzt trinken</v>
+        <v>2021 - 2029</v>
       </c>
       <c r="C146" t="str">
         <v>89/100 (Falstaff)</v>
@@ -3757,7 +3757,7 @@
         <v>€8.90</v>
       </c>
       <c r="E146" t="str">
-        <v>Sauerkirsche, Brombeere &amp; samtiges Tannin</v>
+        <v>0</v>
       </c>
       <c r="F146" t="str">
         <v/>
@@ -3771,7 +3771,7 @@
         <v>Häußermann Spätburgunder Premium 2019 (DE)</v>
       </c>
       <c r="B147" t="str">
-        <v>jetzt trinken</v>
+        <v>2019 - 2027</v>
       </c>
       <c r="C147" t="str">
         <v>1.5* (Eichelmann)</v>
@@ -3780,7 +3780,7 @@
         <v>€12.00</v>
       </c>
       <c r="E147" t="str">
-        <v>samtig, dezent Vanille &amp; Fruchtwucht</v>
+        <v>0</v>
       </c>
       <c r="F147" t="str">
         <v/>
@@ -3794,7 +3794,7 @@
         <v>Rieger Pinot Noir 2023 (DE)</v>
       </c>
       <c r="B148" t="str">
-        <v>jetzt trinken</v>
+        <v>2023 - 2031</v>
       </c>
       <c r="C148" t="str">
         <v>92/100 (Falstaff)</v>
@@ -3803,7 +3803,7 @@
         <v>€10.00</v>
       </c>
       <c r="E148" t="str">
-        <v>Pflaume, Sauerkirsche &amp; Kräuterwürze</v>
+        <v>0</v>
       </c>
       <c r="F148" t="str">
         <v/>
@@ -3826,7 +3826,7 @@
         <v>€7.50</v>
       </c>
       <c r="E149" t="str">
-        <v>Litschi, Stachelbeere &amp; erfrischend</v>
+        <v>0</v>
       </c>
       <c r="F149" t="str">
         <v/>
@@ -3840,7 +3840,7 @@
         <v>Hoffmann Spätburgunder 2022 (DE)</v>
       </c>
       <c r="B150" t="str">
-        <v>jetzt trinken</v>
+        <v>2022 - 2030</v>
       </c>
       <c r="C150" t="str">
         <v>89/100 (Est.)</v>
@@ -3849,7 +3849,7 @@
         <v>€10.00</v>
       </c>
       <c r="E150" t="str">
-        <v>dunkle Beeren, feine Würze &amp; vollmundig</v>
+        <v>0</v>
       </c>
       <c r="F150" t="str">
         <v/>

</xml_diff>

<commit_message>
docs: update workflow docs and sync latest local backup data
</commit_message>
<xml_diff>
--- a/Weinlager_Details.xlsx
+++ b/Weinlager_Details.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G150"/>
+  <dimension ref="A1:G151"/>
   <cols>
     <col min="1" max="1" width="83.83203125" customWidth="1"/>
     <col min="2" max="2" width="17.83203125" customWidth="1"/>
@@ -405,7 +405,7 @@
     <col min="4" max="4" width="8.83203125" customWidth="1"/>
     <col min="5" max="5" width="11.83203125" customWidth="1"/>
     <col min="6" max="6" width="13.83203125" customWidth="1"/>
-    <col min="7" max="7" width="49.83203125" customWidth="1"/>
+    <col min="7" max="7" width="55.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3858,9 +3858,32 @@
         <v>Recht leicht, süffig. wenig Tiefe</v>
       </c>
     </row>
+    <row r="151">
+      <c r="A151" t="str">
+        <v>Dolde Linsenhöfer Spätburgunder Fass 1 2021</v>
+      </c>
+      <c r="B151" t="str">
+        <v>2021 - 2029</v>
+      </c>
+      <c r="C151" t="str">
+        <v>-</v>
+      </c>
+      <c r="D151" t="str">
+        <v>-</v>
+      </c>
+      <c r="E151" t="str">
+        <v>0</v>
+      </c>
+      <c r="F151" t="str">
+        <v/>
+      </c>
+      <c r="G151" t="str">
+        <v>Leicht, relativ säuerlich, nicht sehr komplex, süffig</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G150"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G151"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>